<commit_message>
docs: Test reports for SDK 9.1
Added test reports for SDK 9.1 generated using TPER-Qmetry script

Signed-off-by: Vaibhav Jindal <v-jindal@ti.com>
</commit_message>
<xml_diff>
--- a/docs/test_report/ethfw_testreport_j7200.xlsx
+++ b/docs/test_report/ethfw_testreport_j7200.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Table of Contents" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Script Input Parameters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Test Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Test Percentage Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan | Execution Report" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Template Help" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Template Revision History" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table of Contents" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Script Input Parameters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Percentage Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan | Execution Report" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Help" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Revision History" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="4" name="_xlnm._FilterDatabase">'Test Plan | Execution Report'!$A$1:$U$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Plan | Execution Report'!$A$1:$U$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -95,54 +95,54 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="14">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="2" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="3" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="4" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="5" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="6" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="3" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="7" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="4" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -506,9 +506,9 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="10"/>
-    <col customWidth="1" max="2" min="2" width="35"/>
-    <col customWidth="1" max="3" min="3" width="80"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -658,10 +658,10 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -674,9 +674,9 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="35"/>
-    <col customWidth="1" max="2" min="2" width="35"/>
-    <col customWidth="1" max="3" min="3" width="35"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -709,12 +709,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2023-11-28 19:16:11.645889-06:00 CDT</t>
+          <t>2023-11-30 23:34:47.895143-06:00 CDT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -727,13 +727,13 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="26"/>
-    <col customWidth="1" max="2" min="2" width="26"/>
-    <col customWidth="1" max="3" min="3" width="26"/>
-    <col customWidth="1" max="4" min="4" width="26"/>
-    <col customWidth="1" max="5" min="5" width="26"/>
-    <col customWidth="1" max="6" min="6" width="26"/>
-    <col customWidth="1" max="7" min="7" width="26"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -791,7 +791,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1028,12 +1028,12 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>76</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1046,12 +1046,12 @@
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="26"/>
-    <col customWidth="1" max="2" min="2" width="26"/>
-    <col customWidth="1" max="3" min="3" width="26"/>
-    <col customWidth="1" max="4" min="4" width="26"/>
-    <col customWidth="1" max="5" min="5" width="26"/>
-    <col customWidth="1" max="6" min="6" width="26"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1289,30 +1289,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U76"/>
+  <dimension ref="A1:U77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="17"/>
-    <col customWidth="1" max="2" min="2" width="24"/>
-    <col customWidth="1" max="3" min="3" width="17"/>
-    <col customWidth="1" max="4" min="4" width="24"/>
-    <col customWidth="1" max="5" min="5" width="17"/>
-    <col customWidth="1" max="6" min="6" width="32"/>
-    <col customWidth="1" max="7" min="7" width="17"/>
-    <col customWidth="1" max="8" min="8" width="17"/>
-    <col customWidth="1" max="9" min="9" width="32"/>
-    <col customWidth="1" max="10" min="10" width="22"/>
-    <col customWidth="1" max="11" min="11" width="32"/>
-    <col customWidth="1" max="12" min="12" width="17"/>
-    <col customWidth="1" max="13" min="13" width="17"/>
-    <col customWidth="1" max="14" min="14" width="17"/>
-    <col customWidth="1" max="15" min="15" width="17"/>
-    <col customWidth="1" max="16" min="16" width="17"/>
-    <col customWidth="1" max="17" min="17" width="17"/>
-    <col customWidth="1" max="18" min="18" width="17"/>
-    <col customWidth="1" max="19" min="19" width="17"/>
-    <col customWidth="1" max="20" min="20" width="24"/>
-    <col customWidth="1" max="21" min="21" width="17"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1470,8 +1470,8 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
-- J7200 EVM with QSGMII expansion card
+          <t>- J7 EVM with GESI expansion card
+- J7200 EVM with QSGMII expansion card
 - J784S4 EVM with QSGMII expansion card</t>
         </is>
       </c>
@@ -1571,8 +1571,8 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
-- J7200 EVM with QSGMII expansion card
+          <t>- J7 EVM with GESI expansion card
+- J7200 EVM with QSGMII expansion card
 - J784S4 EVM with QSGMII expansion card</t>
         </is>
       </c>
@@ -1667,14 +1667,14 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>SafeRTOS cores (MCU2_0 and MCU2_1) running Ethernet firmware should be able to send and receive packets through TCP/UDP/ICMP/IP using integrated inter-core Ethernet driver and lwIP bridge.
-This is demonstrated by running EthFW server and client on R5F0 and R5F1 respectively and making sure that EthFW client on R5F1 is able to get IP address assigned by the external DHCP server.
+          <t>SafeRTOS cores (MCU2_0 and MCU2_1) running Ethernet firmware should be able to send and receive packets through TCP/UDP/ICMP/IP using integrated inter-core Ethernet driver and lwIP bridge.
+This is demonstrated by running EthFW server and client on R5F0 and R5F1 respectively and making sure that EthFW client on R5F1 is able to get IP address assigned by the external DHCP server.
 This process involves broadcast packets (DHCP discover, ARP broadcast ) from the R5F1 client to be routed through the client and server lwIP bridge and inter-core drivers to the external DHCP server thus verifying inter-core Ethernet communication between RTOS cores.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>- J721E EVM, J7200 EVM or J784S4 EVM
+          <t>- J721E EVM, J7200 EVM or J784S4 EVM
 - Linux PC</t>
         </is>
       </c>
@@ -1769,13 +1769,13 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The tap device on A72 Linux, which is created by running the Tap application provided in the SDK, should be able able to send and receive packets with and external PC as well as R5F cores through TCP/UDP/ICMP/IP via inter-core Ethernet and lwIP bridge integrated in the EthFW server on R5F0.
+          <t>The tap device on A72 Linux, which is created by running the Tap application provided in the SDK, should be able able to send and receive packets with and external PC as well as R5F cores through TCP/UDP/ICMP/IP via inter-core Ethernet and lwIP bridge integrated in the EthFW server on R5F0.
 This is demonstrated by running EthFW server and Tap application on R5F0 and A72 Linux respectively, and making sure that Tap device on A72 Linux is able to get IP address assigned by the external DHCP server and ping both the RTOS cores as well using their respective IP addresses.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>- J721E EVM, J7200 EVM or J784S4 EVM.
+          <t>- J721E EVM, J7200 EVM or J784S4 EVM.
 - Linux PC</t>
         </is>
       </c>
@@ -1875,8 +1875,8 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
-- J7200 EVM with QSGMII expansion card
+          <t>- J7 EVM with GESI expansion card
+- J7200 EVM with QSGMII expansion card
 - J784S4 EVM with QSGMII expansion card</t>
         </is>
       </c>
@@ -1976,8 +1976,8 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
-- J7200 EVM with QSGMII expansion card
+          <t>- J7 EVM with GESI expansion card
+- J7200 EVM with QSGMII expansion card
 -J784S4 EVM with QSGMII expansion card</t>
         </is>
       </c>
@@ -2077,8 +2077,8 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
-- J7200 EVM with QSGMII expansion card
+          <t>- J7 EVM with GESI expansion card
+- J7200 EVM with QSGMII expansion card
 - J784S4 EVM with QSGMII expansion card</t>
         </is>
       </c>
@@ -2178,8 +2178,8 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
-- J7200 EVM with QSGMII expansion card
+          <t>- J7 EVM with GESI expansion card
+- J7200 EVM with QSGMII expansion card
 - J784S4 EVM with QSGMII expansion card</t>
         </is>
       </c>
@@ -2279,8 +2279,8 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
-- J7200 EVM with QSGMII expansion card
+          <t>- J7 EVM with GESI expansion card
+- J7200 EVM with QSGMII expansion card
 - J784S4 EVM with QSGMII expansion card</t>
         </is>
       </c>
@@ -2380,8 +2380,8 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
-- J7200 EVM with QSGMII expansion card
+          <t>- J7 EVM with GESI expansion card
+- J7200 EVM with QSGMII expansion card
 - J784S4 EVM with QSGMII expansion card</t>
         </is>
       </c>
@@ -2481,13 +2481,13 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM with GESI expansion card
+          <t>- J7 EVM with GESI expansion card
 - J7200 EVM with QSGMII expansion card</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>1. An ALE policer should be created for remote core's flowIdx for exclusive multicast request.
+          <t>1. An ALE policer should be created for remote core's flowIdx for exclusive multicast request.
 2. Shared multicast requests should result in an update of EthFw's bridge FDB.</t>
         </is>
       </c>
@@ -2577,13 +2577,13 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The tap device on A72 Linux, which is created by running the Tap application provided in the SDK, should be able able to send and receive packets with and external PC as well as R5F cores through TCP/UDP/ICMP/IP via inter-core Ethernet and lwIP bridge integrated in the EthFW server on R5F0.
+          <t>The tap device on A72 Linux, which is created by running the Tap application provided in the SDK, should be able able to send and receive packets with and external PC as well as R5F cores through TCP/UDP/ICMP/IP via inter-core Ethernet and lwIP bridge integrated in the EthFW server on R5F0.
 This is demonstrated by running EthFW server and Tap application on R5F0 and A72 Linux respectively, and making sure that Tap device on A72 Linux is able to get IP address assigned by the external DHCP server and ping both the RTOS cores as well using their respective IP addresses.</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>- J721E EVM, J7200 EVM or J784S4 EVM.
+          <t>- J721E EVM, J7200 EVM or J784S4 EVM.
 - Linux PC</t>
         </is>
       </c>
@@ -2678,14 +2678,14 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>RTOS cores (MCU2_0 and MCU2_1) running Ethernet firmware should be able to send and receive packets through TCP/UDP/ICMP/IP using integrated inter-core Ethernet driver and lwIP bridge.
-This is demonstrated by running EthFW server and client on R5F0 and R5F1 respectively and making sure that EthFW client on R5F1 is able to get IP address assigned by the external DHCP server.
+          <t>RTOS cores (MCU2_0 and MCU2_1) running Ethernet firmware should be able to send and receive packets through TCP/UDP/ICMP/IP using integrated inter-core Ethernet driver and lwIP bridge.
+This is demonstrated by running EthFW server and client on R5F0 and R5F1 respectively and making sure that EthFW client on R5F1 is able to get IP address assigned by the external DHCP server.
 This process involves broadcast packets (DHCP discover, ARP broadcast ) from the R5F1 client to be routed through the client and server lwIP bridge and inter-core drivers to the external DHCP server thus verifying inter-core Ethernet communication between RTOS cores.</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>J721E EVM or J7200 EVM
+          <t>J721E EVM or J7200 EVM
 Linux PC</t>
         </is>
       </c>
@@ -2740,22 +2740,22 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2369</t>
+          <t>ETHFW-2370</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>ETHFW Demo Test Plan</t>
+          <t>ETHFW Thin Clients Test Plan</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1932</t>
+          <t>ETHFW-2537</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Demo: Hardware interVLAN</t>
+          <t>ETHFW: Promiscuous mode on MAC-only port (Linux)</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -2765,34 +2765,33 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-903</t>
+          <t>ETHFW-1711</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>j721e-evm,j7200-evm</t>
+          <t>j721e-evm,j7200-evm,j784s4-evm</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Steps are documented in Ethernet Firmware Demo page: [https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html#ethfw_hw_intervlan_routing]</t>
+          <t>Test that CPSW ALE can be set in promiscuous mode and that all traffic is forwarded to the host port.</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>J721E or J7200 with Ethernet cables connected as follows:
-- J721E: MAC ports 3 and 8
-- J7200: MAC ports 2 and 3</t>
+          <t>J721E/J7200/J784S4 EVM
+Linux PC</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware shall route packets across VLANs in hardware.</t>
+          <t>Ping/Iperf should work fine</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -2802,7 +2801,7 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>Use Case Analysis</t>
+          <t>Requirements-Analysis</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
@@ -2830,11 +2829,19 @@
           <t>ETHFW 9.1 Release Test Run (j7200)</t>
         </is>
       </c>
-      <c r="S15" s="3" t="inlineStr"/>
-      <c r="T15" s="3" t="inlineStr"/>
-      <c r="U15" s="9" t="inlineStr">
-        <is>
-          <t>Pass</t>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2536</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>VLAN tagged packets coming on MAC-only port in promiscuous mode</t>
+        </is>
+      </c>
+      <c r="U15" s="10" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>
@@ -2851,12 +2858,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1931</t>
+          <t>ETHFW-1932</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Demo: IP Next Header Filtering</t>
+          <t>EthFw: Demo: Hardware interVLAN</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -2881,20 +2888,19 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>This demo white-lists TCP and UDP protocols and hence blocking packets of other protocols in the VLAN network.
-Steps are documented in Ethernet Firmware Demo page: [https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html#ethfw_ip_nxthdr_filtering]</t>
+          <t>Steps are documented in Ethernet Firmware Demo page: [https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html#ethfw_hw_intervlan_routing]</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>J721E or J7200 with Ethernet cables connected as follows:
-- J721E: MAC ports 3 and 8
+          <t>J721E or J7200 with Ethernet cables connected as follows:
+- J721E: MAC ports 3 and 8
 - J7200: MAC ports 2 and 3</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Switch should synchronize with PTP master.</t>
+          <t>Ethernet Firmware shall route packets across VLANs in hardware.</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -2953,12 +2959,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1930</t>
+          <t>ETHFW-1931</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Demo: Software interVLAN</t>
+          <t>EthFw: Demo: IP Next Header Filtering</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -2983,19 +2989,20 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Steps are documented in Ethernet Firmware Demo page: [https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html#ethfw_sw_intervlan_routing]</t>
+          <t>This demo white-lists TCP and UDP protocols and hence blocking packets of other protocols in the VLAN network.
+Steps are documented in Ethernet Firmware Demo page: [https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html#ethfw_ip_nxthdr_filtering]</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>J721E or J7200 with Ethernet cables connected as follows:
-- J721E: MAC ports 3 and 8
+          <t>J721E or J7200 with Ethernet cables connected as follows:
+- J721E: MAC ports 3 and 8
 - J7200: MAC ports 2 and 3</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware shall route packets across VLANs in software.</t>
+          <t>Ethernet Switch should synchronize with PTP master.</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -3054,12 +3061,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1928</t>
+          <t>ETHFW-1930</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Demo: PTP stack</t>
+          <t>EthFw: Demo: Software interVLAN</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -3084,18 +3091,19 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Validate PTP stack integration in Ethernet Firmware.
-Steps are documented in Ethernet Firmware Demo page: https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html#demo_ethfw_ptp_stack</t>
+          <t>Steps are documented in Ethernet Firmware Demo page: [https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html#ethfw_sw_intervlan_routing]</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>J721E or J7200 with Ethernet cable connected to a PTP capable device on MAC port 3.</t>
+          <t>J721E or J7200 with Ethernet cables connected as follows:
+- J721E: MAC ports 3 and 8
+- J7200: MAC ports 2 and 3</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Switch should synchronize with PTP master.</t>
+          <t>Ethernet Firmware shall route packets across VLANs in software.</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
@@ -3154,12 +3162,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1927</t>
+          <t>ETHFW-1928</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Demo: Rate limiting</t>
+          <t>EthFw: Demo: PTP stack</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -3184,21 +3192,18 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Validate ALE-based rate limiting feature in Ethernet Firmware.
-Rate Limiting can be enabled by adding a policer entry with parameters like Source and Destination MAC address of the traffic to be limited. The rate at which the traffic is limited is based on the values of Peak Information Rate (PIR) and Committed Information Rate (CIR) both in bits per second (bps) set in the policer entry.
-Steps are documented in Ethernet Firmware Demo page: https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html</t>
+          <t>Validate PTP stack integration in Ethernet Firmware.
+Steps are documented in Ethernet Firmware Demo page: https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html#demo_ethfw_ptp_stack</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>J721E or J7200 with Ethernet cables connected as follows:
-- J721E: MAC ports 3 and 8
-- J7200: MAC ports 2 and 3</t>
+          <t>J721E or J7200 with Ethernet cable connected to a PTP capable device on MAC port 3.</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Packet rate should be rate limited as per test parameters.</t>
+          <t>Ethernet Switch should synchronize with PTP master.</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
@@ -3236,19 +3241,11 @@
           <t>ETHFW 9.1 Release Test Run (j7200)</t>
         </is>
       </c>
-      <c r="S19" s="3" t="inlineStr">
-        <is>
-          <t>ETHFW-791</t>
-        </is>
-      </c>
-      <c r="T19" s="3" t="inlineStr">
-        <is>
-          <t>Rate limiting does not match configured PIR</t>
-        </is>
-      </c>
-      <c r="U19" s="10" t="inlineStr">
-        <is>
-          <t>Fail</t>
+      <c r="S19" s="3" t="inlineStr"/>
+      <c r="T19" s="3" t="inlineStr"/>
+      <c r="U19" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -3265,22 +3262,22 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1664</t>
+          <t>ETHFW-1927</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">[EthFw demos]SW InterVLAN routing </t>
+          <t>EthFw: Demo: Rate limiting</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1179,ETHFW-1244</t>
+          <t>ETHFW-903</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -3290,25 +3287,26 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Run SW InterVLAN routing with GESI/QSGMII ports.
-Demonstrate performance w.r.t. below params
- # Packet per second
- # CPU load</t>
+          <t>Validate ALE-based rate limiting feature in Ethernet Firmware.
+Rate Limiting can be enabled by adding a policer entry with parameters like Source and Destination MAC address of the traffic to be limited. The rate at which the traffic is limited is based on the values of Peak Information Rate (PIR) and Committed Information Rate (CIR) both in bits per second (bps) set in the policer entry.
+Steps are documented in Ethernet Firmware Demo page: https://software-dl.ti.com/jacinto7/esd/processor-sdk-rtos-jacinto7/latest/exports/docs/ethfw/docs/user_guide/demo_ethfw_combined_top.html</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>J7 EVM with GESI Expansion card</t>
+          <t>J721E or J7200 with Ethernet cables connected as follows:
+- J721E: MAC ports 3 and 8
+- J7200: MAC ports 2 and 3</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware should run InterVLAN routing demo and route packet successfully</t>
+          <t>Packet rate should be rate limited as per test parameters.</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
@@ -3318,7 +3316,7 @@
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>Requirements-Analysis</t>
+          <t>Use Case Analysis</t>
         </is>
       </c>
       <c r="N20" s="3" t="inlineStr">
@@ -3346,43 +3344,51 @@
           <t>ETHFW 9.1 Release Test Run (j7200)</t>
         </is>
       </c>
-      <c r="S20" s="3" t="inlineStr"/>
-      <c r="T20" s="3" t="inlineStr"/>
-      <c r="U20" s="9" t="inlineStr">
-        <is>
-          <t>Pass</t>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-791</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>Rate limiting does not match configured PIR</t>
+        </is>
+      </c>
+      <c r="U20" s="10" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2368</t>
+          <t>ETHFW-2369</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>ETHFW Performance Test Plan</t>
+          <t>ETHFW Demo Test Plan</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1419</t>
+          <t>ETHFW-1664</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN stripping</t>
+          <t xml:space="preserve">[EthFw demos]SW InterVLAN routing </t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Requirement</t>
+          <t>Requirement,Requirement</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1255</t>
+          <t>ETHFW-1179,ETHFW-1244</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -3397,7 +3403,10 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN stripping</t>
+          <t>Run SW InterVLAN routing with GESI/QSGMII ports.
+Demonstrate performance w.r.t. below params
+ # Packet per second
+ # CPU load</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -3407,12 +3416,12 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Wire rate switching  for all frame sizes with VLAN stripping should be under acceptable criteria</t>
+          <t>Ethernet Firmware should run InterVLAN routing demo and route packet successfully</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
@@ -3466,12 +3475,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1401</t>
+          <t>ETHFW-1419</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Performance]Switching Performance:Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8</t>
+          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN stripping</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -3481,7 +3490,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1232</t>
+          <t>ETHFW-1255</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -3496,7 +3505,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Switching Performance:Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8 (priority remapping)</t>
+          <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN stripping</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
@@ -3506,7 +3515,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8 (priority remapping) should be under acceptable criteria</t>
+          <t>Wire rate switching  for all frame sizes with VLAN stripping should be under acceptable criteria</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
@@ -3565,12 +3574,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1399</t>
+          <t>ETHFW-1401</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port</t>
+          <t>[EthFW][Performance]Switching Performance:Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -3580,7 +3589,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1196</t>
+          <t>ETHFW-1232</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -3595,7 +3604,7 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port</t>
+          <t>Switching Performance:Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8 (priority remapping)</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -3605,7 +3614,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port should be under acceptable criteria</t>
+          <t>Wire rate switching from ingress queue 1 - 8 to egress queue 1 - 8 (priority remapping) should be under acceptable criteria</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
@@ -3664,12 +3673,12 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1362</t>
+          <t>ETHFW-1399</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN insertion</t>
+          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -3679,7 +3688,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1154</t>
+          <t>ETHFW-1196</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -3694,7 +3703,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN insertion</t>
+          <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -3704,7 +3713,7 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Wire rate switching  for all frame sizes with VLAN insertion should be under acceptable criteria</t>
+          <t>Wire rate switching  for all frame sizes with VLAN modification from ingress to egress port should be under acceptable criteria</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
@@ -3763,12 +3772,12 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1342</t>
+          <t>ETHFW-1362</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes without VLAN.</t>
+          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN insertion</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -3778,7 +3787,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1277</t>
+          <t>ETHFW-1154</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -3793,7 +3802,7 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Switching Performance:Wire rate switching  for all frame sizes without VLAN.</t>
+          <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN insertion</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
@@ -3803,7 +3812,7 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Wire rate switching  for all frame sizes without VLAN should be under acceptable criteria</t>
+          <t>Wire rate switching  for all frame sizes with VLAN insertion should be under acceptable criteria</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
@@ -3862,12 +3871,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1330</t>
+          <t>ETHFW-1342</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">[EthFW][Performance]Switching Performance:Head of line blocking test </t>
+          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes without VLAN.</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -3877,7 +3886,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1170</t>
+          <t>ETHFW-1277</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -3892,8 +3901,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perform multicast and unicast tests to confirm HOL (head of line) blocking doesn't exist in switching
-</t>
+          <t>Switching Performance:Wire rate switching  for all frame sizes without VLAN.</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -3903,7 +3911,7 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>HOL (head of line) blocking doesn't exist in switching</t>
+          <t>Wire rate switching  for all frame sizes without VLAN should be under acceptable criteria</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
@@ -3962,12 +3970,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1323</t>
+          <t>ETHFW-1330</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Performance]Switching Performance:Wire rate broadcast/Multicast traffic</t>
+          <t xml:space="preserve">[EthFW][Performance]Switching Performance:Head of line blocking test </t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -3977,7 +3985,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1302</t>
+          <t>ETHFW-1170</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -3992,7 +4000,8 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Switching Performance:Wire rate broadcast/Multicast traffic</t>
+          <t xml:space="preserve">Perform multicast and unicast tests to confirm HOL (head of line) blocking doesn't exist in switching
+</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -4002,7 +4011,7 @@
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>Wire rate broadcast/Multicast traffic should be under acceptable criteria</t>
+          <t>HOL (head of line) blocking doesn't exist in switching</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
@@ -4061,12 +4070,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1326</t>
+          <t>ETHFW-1323</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN (no packet modification)</t>
+          <t>[EthFW][Performance]Switching Performance:Wire rate broadcast/Multicast traffic</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -4076,7 +4085,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1110</t>
+          <t>ETHFW-1302</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -4091,7 +4100,7 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN (no packet modification)</t>
+          <t>Switching Performance:Wire rate broadcast/Multicast traffic</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
@@ -4101,7 +4110,7 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Wire rate switching  for all frame sizes with VLAN should be under acceptable criteria</t>
+          <t>Wire rate broadcast/Multicast traffic should be under acceptable criteria</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
@@ -4150,71 +4159,62 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2283</t>
+          <t>ETHFW-2368</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>EthFw gPTP Test Plan</t>
+          <t>ETHFW Performance Test Plan</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2274</t>
+          <t>ETHFW-1326</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>EthFw: TSN: gPTP: Master mode</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
+          <t>[EthFW][Performance]Switching Performance:Wire rate switching  for all frame sizes with VLAN (no packet modification)</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-1110</t>
+        </is>
+      </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>j721e-evm,j7200-evm,j784s4-evm</t>
+          <t>j721e-evm,j7200-evm</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Verify that gPTP stack integrated in ETHFW can run as master.
-Testing between two EVMs: (Recommended)
- # Force ETHFW gPTP (DUT) to run as master set CONF_PRIMARY_PRIORITY1 240 using gptpconf_set_item(). If not forcing DUT to be master, DUT can be master/slave.
- # Connect DUT to another EVM running ETHFW example via MAC port 3 on both boards.
-                                                                                 OR
-Testing between EVM and a PC: (Recommended on Intel i210 card)
-        1. Configure gptp2.conf CONF_PRIMARY_PRIORITY1 255 to make PC become slave.
-        2. Run gptp2d on the PC side.
-        3. Check the log from DUT (master) and PC (slave).
-Master logs:
-{code:java}
-GM changed old=00:00:00:00:00:00:00:00, new=70:FF:76:FF:FE:1D:E1:A0{code}
-{code:java}
-domain=0, offset=0nsec, hw-adjrate=0ppb
-            gmsync=true, last_setts64=0nsec ..{code}</t>
+          <t>Switching Performance:Wire rate switching  for all frame sizes with VLAN (no packet modification)</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>1. Force ETHFW gPTP to run as master by setting CONF_PRIMARY_PRIORITY1 240 using gptpconf_set_item(). If DUT is not forced as master, it could run as either master or slave depending on the connected device.
-2. Connect DUT to another EVM running ETHFW example via MAC port 3 on both boards.</t>
+          <t>J7 EVM with GESI Expansion card</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>"GM changed old=00:00:00:00:00:00:00:00, new=70:FF:76:FF:FE:1D:E1:A0"
-domain=0, offset=0nsec, hw-adjrate=0ppb
-            gmsync=true, last_setts64=0nsec ..</t>
+          <t>Wire rate switching  for all frame sizes with VLAN should be under acceptable criteria</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Regression,Sanity</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="P29" s="3" t="inlineStr">
@@ -4268,12 +4268,12 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2282</t>
+          <t>ETHFW-2274</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>EthFw: TSN: gPTP: Slave mode</t>
+          <t>EthFw: TSN: gPTP: Master mode</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr"/>
@@ -4290,36 +4290,34 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Verify that gPTP stack integrated in ETHFW can run as slave.
-Testing between two EVMs: (Recommended)
- # Force ETHFW gPTP (DUT) to run as slave by setting CONF_PRIMARY_PRIORITY1 255 using gptpconf_set_item().
- ## If not forcing DUT to be slave, DUT can be master or slave.
- # Connect DUT to another EVM running ETHFW example via MAC port 3 on both boards.
-                                                                                             OR
-Testing between EVM and PC: (Recommended on Intel i210 card)
-        1. Configure gptp2.conf CONF_PRIMARY_PRIORITY1 240 to make PC become master.
-        2. Run gptp2d on the PC side
-        3. Check the log from DUT (slave) and PC(master)
-Slave logs (when second EVM becomes new GM):
-{code:java}
-GM changed old=24:76:25:FF:FE:96:6C:41, new=70:FF:76:FF:FE:1D:9B:77{code}
-here the machine with MAC address: 70:FF:76:FF:FE:1D:9B:77 is the master
-After a while, DUT will keep printing repeatedly the clock rate without switching GM:
-{code:java}
-INF:gptp:domainNumber=0, clock_master_sync_receive:the master clock rate to &lt;number&gt;ppb{code}</t>
+          <t>Verify that gPTP stack integrated in ETHFW can run as master.
+Testing between two EVMs: (Recommended)
+ # Force ETHFW gPTP (DUT) to run as master set CONF_PRIMARY_PRIORITY1 240 using gptpconf_set_item(). If not forcing DUT to be master, DUT can be master/slave.
+ # Connect DUT to another EVM running ETHFW example via MAC port 3 on both boards.
+                                                                                 OR
+Testing between EVM and a PC: (Recommended on Intel i210 card)
+        1. Configure gptp2.conf CONF_PRIMARY_PRIORITY1 255 to make PC become slave.
+        2. Run gptp2d on the PC side.
+        3. Check the log from DUT (master) and PC (slave).
+Master logs:
+{code:java}
+GM changed old=00:00:00:00:00:00:00:00, new=70:FF:76:FF:FE:1D:E1:A0{code}
+{code:java}
+domain=0, offset=0nsec, hw-adjrate=0ppb
+            gmsync=true, last_setts64=0nsec ..{code}</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>1. Force ETHFW gPTP (DUT) to run as slave set CONF_PRIMARY_PRIORITY1 255 using gptpconf_set_item(). 3. If not forcing DUT to be slave, DUT can be master/slave.
+          <t>1. Force ETHFW gPTP to run as master by setting CONF_PRIMARY_PRIORITY1 240 using gptpconf_set_item(). If DUT is not forced as master, it could run as either master or slave depending on the connected device.
 2. Connect DUT to another EVM running ETHFW example via MAC port 3 on both boards.</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>1. When DUT switches roles from GM to slave, DUT logs should show "GM changed old=24:76:25:FF:FE:96:6C:41, new=70:FF:76:FF:FE:1D:9B:77". Here new GM's MAC address is: 70:FF:76:FF:FE:1D:9B:77.
-2. After a while, DUT will keep printing repeatedly the clock rate without switching GM:  "INF:gptp:domainNumber=0, clock_master_sync_receive:the master clock rate to &lt;number&gt;ppb"
-3. PC will not show clock rate adjustment log.</t>
+          <t>"GM changed old=00:00:00:00:00:00:00:00, new=70:FF:76:FF:FE:1D:E1:A0"
+domain=0, offset=0nsec, hw-adjrate=0ppb
+            gmsync=true, last_setts64=0nsec ..</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
@@ -4378,12 +4376,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2275</t>
+          <t>ETHFW-2282</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>EthFw: TSN: gPTP: Master-slave reliability</t>
+          <t>EthFw: TSN: gPTP: Slave mode</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr"/>
@@ -4400,20 +4398,36 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>1. Keep master (ETHFW-2274) and slave (ETHFW-2282) running 2 hours
-2. Check if the DUT is crashed or not</t>
+          <t>Verify that gPTP stack integrated in ETHFW can run as slave.
+Testing between two EVMs: (Recommended)
+ # Force ETHFW gPTP (DUT) to run as slave by setting CONF_PRIMARY_PRIORITY1 255 using gptpconf_set_item().
+ ## If not forcing DUT to be slave, DUT can be master or slave.
+ # Connect DUT to another EVM running ETHFW example via MAC port 3 on both boards.
+                                                                                             OR
+Testing between EVM and PC: (Recommended on Intel i210 card)
+        1. Configure gptp2.conf CONF_PRIMARY_PRIORITY1 240 to make PC become master.
+        2. Run gptp2d on the PC side
+        3. Check the log from DUT (slave) and PC(master)
+Slave logs (when second EVM becomes new GM):
+{code:java}
+GM changed old=24:76:25:FF:FE:96:6C:41, new=70:FF:76:FF:FE:1D:9B:77{code}
+here the machine with MAC address: 70:FF:76:FF:FE:1D:9B:77 is the master
+After a while, DUT will keep printing repeatedly the clock rate without switching GM:
+{code:java}
+INF:gptp:domainNumber=0, clock_master_sync_receive:the master clock rate to &lt;number&gt;ppb{code}</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Connect two devices running ETHFW, one device as master and another as slave.
-For the device in master mode, refer to test setup instructions in ETHFW-2274.
-For the device in slave mode, refer to test setup instructions in ETHFW-2282.</t>
+          <t>1. Force ETHFW gPTP (DUT) to run as slave set CONF_PRIMARY_PRIORITY1 255 using gptpconf_set_item(). 3. If not forcing DUT to be slave, DUT can be master/slave.
+2. Connect DUT to another EVM running ETHFW example via MAC port 3 on both boards.</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>ETHFW application continues to run properly and the two devices (master and slave) are still synchronized.</t>
+          <t>1. When DUT switches roles from GM to slave, DUT logs should show "GM changed old=24:76:25:FF:FE:96:6C:41, new=70:FF:76:FF:FE:1D:9B:77". Here new GM's MAC address is: 70:FF:76:FF:FE:1D:9B:77.
+2. After a while, DUT will keep printing repeatedly the clock rate without switching GM:  "INF:gptp:domainNumber=0, clock_master_sync_receive:the master clock rate to &lt;number&gt;ppb"
+3. PC will not show clock rate adjustment log.</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
@@ -4472,12 +4486,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2281</t>
+          <t>ETHFW-2275</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>EthFw: TSN: gPTP: Disconnect/re-connect in master mode</t>
+          <t>EthFw: TSN: gPTP: Master-slave reliability</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr"/>
@@ -4494,19 +4508,20 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Verifies that gPTP stack integrated in ETHFW continues to work properly as a master after cable disconnect/reconnect, and synchronize with the connected device.</t>
+          <t>1. Keep master (ETHFW-2274) and slave (ETHFW-2282) running 2 hours
+2. Check if the DUT is crashed or not</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Refer to ETHFW slave test setup described in ETHFW-2274.</t>
+          <t>Connect two devices running ETHFW, one device as master and another as slave.
+For the device in master mode, refer to test setup instructions in ETHFW-2274.
+For the device in slave mode, refer to test setup instructions in ETHFW-2282.</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>DUT shows the disconnected log like this: "INF:gptp:gptpnet_cb_devdown:portIndex=1", and the clock rate log will disappear on the PC side.
-After reconnecting: DUT show log like this "INF:gptp:index=1 speed=1000, duplex=full, ptpdev=tilld0", and works as master. 
-The result should be as mentioned in ETHFW-2274</t>
+          <t>ETHFW application continues to run properly and the two devices (master and slave) are still synchronized.</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
@@ -4565,12 +4580,12 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2376</t>
+          <t>ETHFW-2281</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>EthFw: TSN: gPTP: Disconnect/re-connected in slave mode</t>
+          <t>EthFw: TSN: gPTP: Disconnect/re-connect in master mode</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr"/>
@@ -4587,18 +4602,19 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Verifies that gPTP stack integrated in ETHFW continues to work properly as slave after cable disconnect/reconnect, and synchronize with the connected device.</t>
+          <t>Verifies that gPTP stack integrated in ETHFW continues to work properly as a master after cable disconnect/reconnect, and synchronize with the connected device.</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>Refer to ETHFW slave test setup described in ETHFW-2282.</t>
+          <t>Refer to ETHFW slave test setup described in ETHFW-2274.</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>DUT shows the disconnected log like this: "INF:gptp:gptpnet_cb_devdown:portIndex=1", and the clock rate log will disappear
-After reconnecting, DUT works as slave and the result should be same as the mentioned in ETHFW-2282.</t>
+          <t>DUT shows the disconnected log like this: "INF:gptp:gptpnet_cb_devdown:portIndex=1", and the clock rate log will disappear on the PC side.
+After reconnecting: DUT show log like this "INF:gptp:index=1 speed=1000, duplex=full, ptpdev=tilld0", and works as master. 
+The result should be as mentioned in ETHFW-2274</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
@@ -4647,34 +4663,26 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2372</t>
+          <t>ETHFW-2283</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 9.x Release Test Plan (j7200)</t>
+          <t>EthFw gPTP Test Plan</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2367</t>
+          <t>ETHFW-2376</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Packaging] TI TSPA License</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Requirement</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>ETHFW-1237</t>
-        </is>
-      </c>
+          <t>EthFw: TSN: gPTP: Disconnect/re-connected in slave mode</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
       <c r="G34" s="3" t="inlineStr">
         <is>
           <t>j721e-evm,j7200-evm,j784s4-evm</t>
@@ -4682,32 +4690,33 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Verify that Ethernet Firmware source files are released under TI Text File License (TSPA).</t>
+          <t>Verifies that gPTP stack integrated in ETHFW continues to work properly as slave after cable disconnect/reconnect, and synchronize with the connected device.</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>ETHFW repository with source code.</t>
+          <t>Refer to ETHFW slave test setup described in ETHFW-2282.</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>All source files shall have TI TSPA license header.</t>
+          <t>DUT shows the disconnected log like this: "INF:gptp:gptpnet_cb_devdown:portIndex=1", and the clock rate log will disappear
+After reconnecting, DUT works as slave and the result should be same as the mentioned in ETHFW-2282.</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>Usability</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>Customer Usage</t>
+          <t>Requirements-Analysis</t>
         </is>
       </c>
       <c r="N34" s="3" t="inlineStr">
@@ -4717,7 +4726,7 @@
       </c>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Regression,Sanity</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">
@@ -4756,12 +4765,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2233</t>
+          <t>ETHFW-2367</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Boot time benchmark</t>
+          <t>[EthFW][Packaging] TI TSPA License</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -4771,7 +4780,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1964</t>
+          <t>ETHFW-1237</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -4786,34 +4795,27 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Test that Linux client application can enable a virtual MAC interface configured in MAC-only mode.</t>
+          <t>Verify that Ethernet Firmware source files are released under TI Text File License (TSPA).</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>EVM #1 running ETHFW should be as follows:
-- J7 EVM with GESI expansion + QSGMII expansion cards
-- J7200 EVM with QSGMII expansion card
-- J784S4 EVM with QSGMII expansion card
-EVM #2 is needed which will run Enet LLD lwIP as described in the following testcases:
-- J721E: See setup in testcase ETHFW-2065.
-- J7200: See setup in testcase ETHFW-2067.
-- J784S4: See setup in testcase ETHFW-2071.</t>
+          <t>ETHFW repository with source code.</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>ETHFW boot time shall be printed in console.</t>
+          <t>All source files shall have TI TSPA license header.</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Usability</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>Requirements-Analysis</t>
+          <t>Customer Usage</t>
         </is>
       </c>
       <c r="N35" s="3" t="inlineStr">
@@ -4862,12 +4864,12 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2124</t>
+          <t>ETHFW-2233</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EthFw: SafeRTOS: Static IP test </t>
+          <t>EthFw: Boot time benchmark</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -4877,7 +4879,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2115</t>
+          <t>ETHFW-1964</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -4892,30 +4894,34 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware built for SafeRTOS with static IP address tests.</t>
+          <t>Test that Linux client application can enable a virtual MAC interface configured in MAC-only mode.</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>- J7 EVM, J7200 EVM or J784S4 EVM
-- GESI board (J721E) or QSGMII board (J7200, J748S4)
-- PC</t>
+          <t>EVM #1 running ETHFW should be as follows:
+- J7 EVM with GESI expansion + QSGMII expansion cards
+- J7200 EVM with QSGMII expansion card
+- J784S4 EVM with QSGMII expansion card
+EVM #2 is needed which will run Enet LLD lwIP as described in the following testcases:
+- J721E: See setup in testcase ETHFW-2065.
+- J7200: See setup in testcase ETHFW-2067.
+- J784S4: See setup in testcase ETHFW-2071.</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>* eth1 interface should get a dynamic IP address and ping to this address should work fine.
-* eth1 interface should be able to pass static IP and ping to this address should work fine.</t>
+          <t>ETHFW boot time shall be printed in console.</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
         <is>
-          <t>Customer Usage</t>
+          <t>Requirements-Analysis</t>
         </is>
       </c>
       <c r="N36" s="3" t="inlineStr">
@@ -4964,22 +4970,22 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2010</t>
+          <t>ETHFW-2124</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Standalone test with CCS boot</t>
+          <t xml:space="preserve">EthFw: SafeRTOS: Static IP test </t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1947,ETHFW-1952</t>
+          <t>ETHFW-2115</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -4994,26 +5000,20 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware should be able to run with CCS boot and enable the MAC ports as follows:
- * J721E: All 8 MAC ports.
- * J7200: All 4 MAC ports.
- * J784S4: 4 MAC ports in QSGMII expansion board + 1 MAC port in bridge board (optional).
- Refer to EthFw User's Guide for port mode allocation (switch mode vs MAC-only mode).
-EthFw shall be able to acquire an IP address from network.</t>
+          <t>Ethernet Firmware built for SafeRTOS with static IP address tests.</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>J721E/J7200/J784S4 EVM
-Linux PC</t>
+          <t>- J7 EVM, J7200 EVM or J784S4 EVM
+- GESI board (J721E) or QSGMII board (J7200, J748S4)
+- PC</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>EthFw should be able to successfully initialize and configure the MAC ports enabled for the given SoC.
-J721E: All 8 MAC ports.
-J7200: All 4 MAC ports.
-J784S4: 4 MAC ports in QSGMII expansion board + 1 MAC port in bridge board (optional).</t>
+          <t>* eth1 interface should get a dynamic IP address and ping to this address should work fine.
+* eth1 interface should be able to pass static IP and ping to this address should work fine.</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t>Requirements-Analysis</t>
+          <t>Customer Usage</t>
         </is>
       </c>
       <c r="N37" s="3" t="inlineStr">
@@ -5072,12 +5072,12 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2009</t>
+          <t>ETHFW-2010</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Standalone test with SBL boot</t>
+          <t>EthFw: Standalone test with CCS boot</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1952,ETHFW-1947</t>
+          <t>ETHFW-1947,ETHFW-1952</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -5102,25 +5102,25 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware should be able to run with SBL boot and enable the MAC ports as follows:
- * J721E: All 8 MAC ports.
- * J7200: All 4 MAC ports.
- * J784S4: 4 MAC ports in QSGMII expansion board + 1 MAC port in bridge board (optional).
- Refer to EthFw User's Guide for port mode allocation (switch mode vs MAC-only mode).
+          <t>Ethernet Firmware should be able to run with CCS boot and enable the MAC ports as follows:
+ * J721E: All 8 MAC ports.
+ * J7200: All 4 MAC ports.
+ * J784S4: 4 MAC ports in QSGMII expansion board + 1 MAC port in bridge board (optional).
+ Refer to EthFw User's Guide for port mode allocation (switch mode vs MAC-only mode).
 EthFw shall be able to acquire an IP address from network.</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>J721E/J7200/J784S4 EVM
+          <t>J721E/J7200/J784S4 EVM
 Linux PC</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>EthFw should be able to successfully initialize and configure the MAC ports enabled for the given SoC.
-J721E: All 8 MAC ports.
-J7200: All 4 MAC ports.
+          <t>EthFw should be able to successfully initialize and configure the MAC ports enabled for the given SoC.
+J721E: All 8 MAC ports.
+J7200: All 4 MAC ports.
 J784S4: 4 MAC ports in QSGMII expansion board + 1 MAC port in bridge board (optional).</t>
         </is>
       </c>
@@ -5180,22 +5180,22 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1823</t>
+          <t>ETHFW-2009</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EthFw: lwIP Integration </t>
+          <t>EthFw: Standalone test with SBL boot</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement,Requirement,Requirement,Requirement,Requirement,Requirement</t>
+          <t>Requirement,Requirement</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1966,ETHFW-1953,ETHFW-1912,ETHFW-1950,ETHFW-1718,ETHFW-1716,ETHFW-1742</t>
+          <t>ETHFW-1952,ETHFW-1947</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -5210,19 +5210,26 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware should be able to send and receive packets through TCP/UDP/ICMP/IP using integrated lwIP stack.
-lwIP integration validation also verifies FreeRTOS integration.</t>
+          <t>Ethernet Firmware should be able to run with SBL boot and enable the MAC ports as follows:
+ * J721E: All 8 MAC ports.
+ * J7200: All 4 MAC ports.
+ * J784S4: 4 MAC ports in QSGMII expansion board + 1 MAC port in bridge board (optional).
+ Refer to EthFw User's Guide for port mode allocation (switch mode vs MAC-only mode).
+EthFw shall be able to acquire an IP address from network.</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>J721E EVM, J7200 EVM or J784S4 EVM
+          <t>J721E/J7200/J784S4 EVM
 Linux PC</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>EthFw should be able to successfully establish a connection with an external device, acquire IP address and exchange packets.</t>
+          <t>EthFw should be able to successfully initialize and configure the MAC ports enabled for the given SoC.
+J721E: All 8 MAC ports.
+J7200: All 4 MAC ports.
+J784S4: 4 MAC ports in QSGMII expansion board + 1 MAC port in bridge board (optional).</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
@@ -5281,27 +5288,27 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1701</t>
+          <t>ETHFW-1823</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>[EthFw] Windows build support</t>
+          <t xml:space="preserve">EthFw: lwIP Integration </t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement</t>
+          <t>Requirement,Requirement,Requirement,Requirement,Requirement,Requirement,Requirement</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1686,ETHFW-1742</t>
+          <t>ETHFW-1966,ETHFW-1953,ETHFW-1912,ETHFW-1950,ETHFW-1718,ETHFW-1716,ETHFW-1742</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>j721e-evm,j7200-evm</t>
+          <t>j721e-evm,j7200-evm,j784s4-evm</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -5311,21 +5318,19 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Build EthFw separately for J7200 and J721E in a Windows PC.</t>
+          <t>Ethernet Firmware should be able to send and receive packets through TCP/UDP/ICMP/IP using integrated lwIP stack.
+lwIP integration validation also verifies FreeRTOS integration.</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>Windows PC and Processor SDK release package.</t>
+          <t>J721E EVM, J7200 EVM or J784S4 EVM
+Linux PC</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>The following EthFw images shall be built:
-* EthFw image for CCS with symbols
-* EthFw image for Linux/QNX with symbols
-* EthFw image for CCS without symbols (_strip.xer5f file)
-* EthFw image for Linux/QNX without symbols (_strip.xer5f file)</t>
+          <t>EthFw should be able to successfully establish a connection with an external device, acquire IP address and exchange packets.</t>
         </is>
       </c>
       <c r="L40" s="3" t="inlineStr">
@@ -5365,9 +5370,9 @@
       </c>
       <c r="S40" s="3" t="inlineStr"/>
       <c r="T40" s="3" t="inlineStr"/>
-      <c r="U40" s="10" t="inlineStr">
-        <is>
-          <t>Fail</t>
+      <c r="U40" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -5384,27 +5389,27 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1552</t>
+          <t>ETHFW-1701</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][System]Protocol: ARP/RARP protocol database: Single Core must maintain ARP entries for MAC/IP address assigned to other cores</t>
+          <t>[EthFw] Windows build support</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Requirement</t>
+          <t>Requirement,Requirement</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1229</t>
+          <t>ETHFW-1686,ETHFW-1742</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>j721e-evm,j7200-evm,j784s4-evm</t>
+          <t>j721e-evm,j7200-evm</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -5414,23 +5419,21 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Protocol: ARP/RARP protocol
- Protocol: ARP/RARP protocol database: Single Core must maintain ARP entries for MAC/IP address assigned to other cores
-In CPSW9G, the broadcast and multicast traffic can be handled by only single core and EthFw handles it. So all broadcast packets are received by only EthFw. Virtual clients only receive unicast packets with MAC address assigned to it.
-Due to this limitation, the ARP requests for remote clients which are broadcast packets can’t be received by remote clients hence it can’t communication with external world.
-To avoid this, remote clients should register their IP with EthFW/R5 which serves the ARP requests on remote clients behalf and EthFw should maintain these ARP entries.
-Now once the external communicating entity has MAC address for QNX, it sends direct unicast packets which are anyway are directly received on remote clients.</t>
+          <t>Build EthFw separately for J7200 and J721E in a Windows PC.</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">J7 EVM with GESI or QSGMII Expansion card
-</t>
+          <t>Windows PC and Processor SDK release package.</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Remote client running on mcu2_1 should be able to register IP address with EthFw. Ping from PC to remote client should work</t>
+          <t>The following EthFw images shall be built:
+* EthFw image for CCS with symbols
+* EthFw image for Linux/QNX with symbols
+* EthFw image for CCS without symbols (_strip.xer5f file)
+* EthFw image for Linux/QNX without symbols (_strip.xer5f file)</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
@@ -5450,7 +5453,7 @@
       </c>
       <c r="O41" s="3" t="inlineStr">
         <is>
-          <t>Regression</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="P41" s="3" t="inlineStr">
@@ -5470,9 +5473,9 @@
       </c>
       <c r="S41" s="3" t="inlineStr"/>
       <c r="T41" s="3" t="inlineStr"/>
-      <c r="U41" s="9" t="inlineStr">
-        <is>
-          <t>Pass</t>
+      <c r="U41" s="10" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>
@@ -5489,12 +5492,12 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1551</t>
+          <t>ETHFW-1552</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Protocol]Protocol: Switch resident protocol:802.1AS rev support</t>
+          <t>[EthFW][System]Protocol: ARP/RARP protocol database: Single Core must maintain ARP entries for MAC/IP address assigned to other cores</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -5504,12 +5507,12 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1293</t>
+          <t>ETHFW-1229</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>j721e-evm,j7200-evm</t>
+          <t>j721e-evm,j7200-evm,j784s4-evm</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -5519,17 +5522,23 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Protocol:802.1AS rev support</t>
+          <t>Protocol: ARP/RARP protocol
+ Protocol: ARP/RARP protocol database: Single Core must maintain ARP entries for MAC/IP address assigned to other cores
+In CPSW9G, the broadcast and multicast traffic can be handled by only single core and EthFw handles it. So all broadcast packets are received by only EthFw. Virtual clients only receive unicast packets with MAC address assigned to it.
+Due to this limitation, the ARP requests for remote clients which are broadcast packets can’t be received by remote clients hence it can’t communication with external world.
+To avoid this, remote clients should register their IP with EthFW/R5 which serves the ARP requests on remote clients behalf and EthFw should maintain these ARP entries.
+Now once the external communicating entity has MAC address for QNX, it sends direct unicast packets which are anyway are directly received on remote clients.</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  J7 EVM with GESI or QSGMII Expansion card </t>
+          <t xml:space="preserve">J7 EVM with GESI or QSGMII Expansion card
+</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>ETHFW running on mcu2_0 should synchronize with Master running on PC</t>
+          <t>Remote client running on mcu2_1 should be able to register IP address with EthFw. Ping from PC to remote client should work</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
@@ -5588,12 +5597,12 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1547</t>
+          <t>ETHFW-1551</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>EthFw - Support EthFw as library to enable SDK integration</t>
+          <t>[EthFW][Protocol]Protocol: Switch resident protocol:802.1AS rev support</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -5603,7 +5612,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1119</t>
+          <t>ETHFW-1293</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -5618,20 +5627,17 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ethfw does not have a unified library interface like EthFw_init() that would pull in all dependent libs and perform system initialization. Such an interface would be required to integrate with vision apps.  
-Currently ethFw is an app enabling basic switching, remote config server for virtual clients etc. with switch config server running for getting configuration from the PC client tool.
-Requirement is to support EthFw as an Library for SDK integration. 
- </t>
+          <t>Protocol:802.1AS rev support</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>J7 EVM with QSGMII or GESI or both daughter boards</t>
+          <t xml:space="preserve">  J7 EVM with GESI or QSGMII Expansion card </t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>EthFw server app should be able to link EthFw library and configure CPSW9G switch.</t>
+          <t>ETHFW running on mcu2_0 should synchronize with Master running on PC</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
@@ -5690,12 +5696,12 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1545</t>
+          <t>ETHFW-1547</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][Linux] Ethfw binary should have fixed UART ID assigned for console output</t>
+          <t>EthFw - Support EthFw as library to enable SDK integration</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -5705,7 +5711,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1253</t>
+          <t>ETHFW-1119</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -5720,21 +5726,20 @@
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Ethfw binary should have fixed UART ID assigned for console output (debugging) for each supported platform.
-It's required for proper DT configuration - UART used by EthFW has to be disabled in DT for Linux.
-j721e - UART 2, serial@2820000</t>
+          <t xml:space="preserve">Ethfw does not have a unified library interface like EthFw_init() that would pull in all dependent libs and perform system initialization. Such an interface would be required to integrate with vision apps.  
+Currently ethFw is an app enabling basic switching, remote config server for virtual clients etc. with switch config server running for getting configuration from the PC client tool.
+Requirement is to support EthFw as an Library for SDK integration. 
+ </t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">mcu2_0  - app_remoteswitchcfg_server.xer5f 
-</t>
+          <t>J7 EVM with QSGMII or GESI or both daughter boards</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EthFw should initialize and print the logs including version info on Main domain UART instance 2 (UART2)
-</t>
+          <t>EthFw server app should be able to link EthFw library and configure CPSW9G switch.</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
@@ -5793,12 +5798,12 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1543</t>
+          <t>ETHFW-1545</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EthFw: Support Thumb2 mode on R5F </t>
+          <t>[EthFw][Linux] Ethfw binary should have fixed UART ID assigned for console output</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -5808,7 +5813,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-761</t>
+          <t>ETHFW-1253</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -5823,29 +5828,21 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>This is a cloned requirement from PRSDK-5804
-Copied description below 
-================
-We have been performing performance benchmarking on R5F using TI ARM compiler on AM65x for Panasonic and broader Motor Drives EE space and have seen R5F performance is significantly better with smaller code size with Thumb2 mode which is a hybrid mode supported on Cortex R5F that generates a mix of 16 bit and 32 bit integers. 
-The TI ARM compiler team that has been support Cortex M and Cortex R devices in connected MCU have recommended use of Thumb2 (code_state=16) instead of ARM mode (code_state=32) and also provide this guidance to customer to optimize Cortex R5 performance.
-[http://processors.wiki.ti.com/index.php/ARM_compiler_optimizations#Tips_for_getting_the_best_performance]
- It appears that current support for PRocessor SDK RTOS software is building all of the R5F code in ARM mode but for non-safety usecases, customer need the option to run code in Thumb2 mode.
-We have performed basic sanity testing of RTOS examples with Thumb2 compiler time option and not seen any functional issues. Can we consider bring this support into PRSDK baseline. 
-*Response from SDO RTOS team for this request:*
-This can be supported. A new Thumb2 R5F target would be required. And we’d have to scrub all existing embedded assembly code to make sure it uses thumb2 instructions
-Discussion with Raghu and Alan DeMars is attached for reference.
-[^RE R5F Compile time flags Thumb2 mode support in TI RTOS for R5F .msg]
-Functional Requirement based on req:CATREQ-2455</t>
+          <t>Ethfw binary should have fixed UART ID assigned for console output (debugging) for each supported platform.
+It's required for proper DT configuration - UART used by EthFW has to be disabled in DT for Linux.
+j721e - UART 2, serial@2820000</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>J7 EVM with QSGMII or GESI or both daughter boards</t>
+          <t xml:space="preserve">mcu2_0  - app_remoteswitchcfg_server.xer5f 
+</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>The app should be able to run without any issue to completion and there should be performance improvement compared to the NON-thumb mode when running the SW inerVLAN routing app</t>
+          <t xml:space="preserve">EthFw should initialize and print the logs including version info on Main domain UART instance 2 (UART2)
+</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
@@ -5904,12 +5901,12 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1542</t>
+          <t>ETHFW-1543</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>[CPSW][System]Timesynch:Forward Timesync event to other registered cores</t>
+          <t xml:space="preserve">EthFw: Support Thumb2 mode on R5F </t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -5919,7 +5916,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1287</t>
+          <t>ETHFW-761</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -5934,17 +5931,29 @@
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Timesynch:Forward Timesync event to other registered cores</t>
+          <t>This is a cloned requirement from PRSDK-5804
+Copied description below 
+================
+We have been performing performance benchmarking on R5F using TI ARM compiler on AM65x for Panasonic and broader Motor Drives EE space and have seen R5F performance is significantly better with smaller code size with Thumb2 mode which is a hybrid mode supported on Cortex R5F that generates a mix of 16 bit and 32 bit integers. 
+The TI ARM compiler team that has been support Cortex M and Cortex R devices in connected MCU have recommended use of Thumb2 (code_state=16) instead of ARM mode (code_state=32) and also provide this guidance to customer to optimize Cortex R5 performance.
+[http://processors.wiki.ti.com/index.php/ARM_compiler_optimizations#Tips_for_getting_the_best_performance]
+ It appears that current support for PRocessor SDK RTOS software is building all of the R5F code in ARM mode but for non-safety usecases, customer need the option to run code in Thumb2 mode.
+We have performed basic sanity testing of RTOS examples with Thumb2 compiler time option and not seen any functional issues. Can we consider bring this support into PRSDK baseline. 
+*Response from SDO RTOS team for this request:*
+This can be supported. A new Thumb2 R5F target would be required. And we’d have to scrub all existing embedded assembly code to make sure it uses thumb2 instructions
+Discussion with Raghu and Alan DeMars is attached for reference.
+[^RE R5F Compile time flags Thumb2 mode support in TI RTOS for R5F .msg]
+Functional Requirement based on req:CATREQ-2455</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> J7 EVM with GESI or QSGMII Expansion card </t>
+          <t>J7 EVM with QSGMII or GESI or both daughter boards</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Remote client running on mcu2_1 should be able to receive CPTS hardware push notifications and able to synchronize with grandmaster using event information.</t>
+          <t>The app should be able to run without any issue to completion and there should be performance improvement compared to the NON-thumb mode when running the SW inerVLAN routing app</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
@@ -6003,12 +6012,12 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1424</t>
+          <t>ETHFW-1542</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>EthFW EMAC OSAL Test - Baremetal implementation</t>
+          <t>[CPSW][System]Timesynch:Forward Timesync event to other registered cores</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -6018,7 +6027,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-941</t>
+          <t>ETHFW-1287</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -6033,17 +6042,17 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][OS]OSAL:EMAC Osal:Baremetal implementation of EMAL osal interface should be integrated into the switch firmware</t>
+          <t>Timesynch:Forward Timesync event to other registered cores</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>J7 EVM with GESI Expansion card</t>
+          <t xml:space="preserve"> J7 EVM with GESI or QSGMII Expansion card </t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Execute cpsw baremetal test app and confirm successful execution</t>
+          <t>Remote client running on mcu2_1 should be able to receive CPTS hardware push notifications and able to synchronize with grandmaster using event information.</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
@@ -6063,7 +6072,7 @@
       </c>
       <c r="O47" s="3" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="P47" s="3" t="inlineStr">
@@ -6102,12 +6111,12 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1415</t>
+          <t>ETHFW-1424</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>EthFW OS Test - CPSW LLD validation</t>
+          <t>EthFW EMAC OSAL Test - Baremetal implementation</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -6117,7 +6126,7 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-903</t>
+          <t>ETHFW-941</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -6132,7 +6141,7 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][OS]OS:cpsw_lld should be validated on split mode variant of TI RTOS config</t>
+          <t>[EthFW][OS]OSAL:EMAC Osal:Baremetal implementation of EMAL osal interface should be integrated into the switch firmware</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
@@ -6142,7 +6151,7 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EthFw switching app should run successfully on MCU_2_1 with MCU _2 configured in split mode </t>
+          <t>Execute cpsw baremetal test app and confirm successful execution</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
@@ -6201,12 +6210,12 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1405</t>
+          <t>ETHFW-1415</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>EthFW System Test - GPTIMER Driver Integration</t>
+          <t>EthFW OS Test - CPSW LLD validation</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -6216,7 +6225,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-955</t>
+          <t>ETHFW-903</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -6231,7 +6240,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][System]Driver Integration:GPTIMER: GPTIMER driver should be integrated</t>
+          <t>[EthFW][OS]OS:cpsw_lld should be validated on split mode variant of TI RTOS config</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
@@ -6241,7 +6250,7 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Confirm packet interrupts occur at periodic 500us interval only when interrupt pacing is enabled. The interrupt pacing is triggered by TImer interrupt</t>
+          <t xml:space="preserve">EthFw switching app should run successfully on MCU_2_1 with MCU _2 configured in split mode </t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
@@ -6300,22 +6309,22 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1355</t>
+          <t>ETHFW-1405</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][Packaging] The ethernet firmware shall be hosted in a separate repo to support firmware only release decoupled from rest of Processor SDK</t>
+          <t>EthFW System Test - GPTIMER Driver Integration</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1290,ETHFW-1135</t>
+          <t>ETHFW-955</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -6330,9 +6339,7 @@
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ethernet firmware shall be hosted in a separate repo to support firmware only release decoupled from rest of Processor SDK
-This will require ethernet firmware to have independent release plan (and version plan) decoupled from Processor SDK PDK
-This is needed to allow LCPD to consume CPSW Ethernet switch firmware without waiting for Processor SDK RTOS  </t>
+          <t>[EthFW][System]Driver Integration:GPTIMER: GPTIMER driver should be integrated</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
@@ -6342,19 +6349,17 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>1. separate package for ethfw
-2. should be available at external git.ti.com
-3. should be released under TI-TFL license</t>
+          <t>Confirm packet interrupts occur at periodic 500us interval only when interrupt pacing is enabled. The interrupt pacing is triggered by TImer interrupt</t>
         </is>
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>Usability</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr">
         <is>
-          <t>Customer Usage</t>
+          <t>Requirements-Analysis</t>
         </is>
       </c>
       <c r="N50" s="3" t="inlineStr">
@@ -6403,22 +6408,22 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1344</t>
+          <t>ETHFW-1355</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>EthFW System Test - PMU Driver Integration</t>
+          <t>[EthFW][Packaging] The ethernet firmware shall be hosted in a separate repo to support firmware only release decoupled from rest of Processor SDK</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Requirement</t>
+          <t>Requirement,Requirement</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-937</t>
+          <t>ETHFW-1290,ETHFW-1135</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -6433,7 +6438,9 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][System]Driver Integration:PMU: PMU driver should be integrated</t>
+          <t xml:space="preserve">The ethernet firmware shall be hosted in a separate repo to support firmware only release decoupled from rest of Processor SDK
+This will require ethernet firmware to have independent release plan (and version plan) decoupled from Processor SDK PDK
+This is needed to allow LCPD to consume CPSW Ethernet switch firmware without waiting for Processor SDK RTOS  </t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
@@ -6443,17 +6450,19 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Should be able to get PMU counters for perfomance profiling</t>
+          <t>1. separate package for ethfw
+2. should be available at external git.ti.com
+3. should be released under TI-TFL license</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Usability</t>
         </is>
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t>Requirements-Analysis</t>
+          <t>Customer Usage</t>
         </is>
       </c>
       <c r="N51" s="3" t="inlineStr">
@@ -6502,22 +6511,22 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1331</t>
+          <t>ETHFW-1344</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][IPC]IPC:All CPSW subsystem register setting shall be done by means of IPC message to switch R5 core.Not direct register config shall be done on remote cores.</t>
+          <t>EthFW System Test - PMU Driver Integration</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1203,ETHFW-2170</t>
+          <t>ETHFW-937</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -6532,17 +6541,17 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>IPC:All CPSW subsystem register setting shall be done by means of IPC message to switch R5 core.Not direct register config shall be done on remote cores.</t>
+          <t>[EthFW][System]Driver Integration:PMU: PMU driver should be integrated</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>J7 EVM with GESI or QSGMII DB</t>
+          <t>J7 EVM with GESI Expansion card</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>&lt;To be updated&gt;</t>
+          <t>Should be able to get PMU counters for perfomance profiling</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
@@ -6562,7 +6571,7 @@
       </c>
       <c r="O52" s="3" t="inlineStr">
         <is>
-          <t>Regression</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="P52" s="3" t="inlineStr">
@@ -6601,22 +6610,22 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1325</t>
+          <t>ETHFW-1331</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>EthFW System Test - TISCI client Driver Integration</t>
+          <t>[EthFw][IPC]IPC:All CPSW subsystem register setting shall be done by means of IPC message to switch R5 core.Not direct register config shall be done on remote cores.</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Requirement</t>
+          <t>Requirement,Requirement</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-899</t>
+          <t>ETHFW-1203,ETHFW-2170</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -6631,17 +6640,17 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>[EthFW][System]Driver Integration:TISCI: TISCI client driver should be integrated for DMSC IPC</t>
+          <t>IPC:All CPSW subsystem register setting shall be done by means of IPC message to switch R5 core.Not direct register config shall be done on remote cores.</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>J7 EVM with GESI Expansion card</t>
+          <t>J7 EVM with GESI or QSGMII DB</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirm successful execution with DMSC firmware </t>
+          <t>&lt;To be updated&gt;</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
@@ -6661,7 +6670,7 @@
       </c>
       <c r="O53" s="3" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="P53" s="3" t="inlineStr">
@@ -6700,22 +6709,22 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1097</t>
+          <t>ETHFW-1325</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][IPC]IPC: Support for remote core to query if switch R5 firmware has been loaded</t>
+          <t>EthFW System Test - TISCI client Driver Integration</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1184,ETHFW-2172</t>
+          <t>ETHFW-899</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -6730,7 +6739,7 @@
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>For generic kernel driver in mainline, dependency on pre-initialization is not good experience (people use different bootloader, boot sequence etc). So there should be a way to query of firmware is loaded and if not let driver load it from filesystem.</t>
+          <t>[EthFW][System]Driver Integration:TISCI: TISCI client driver should be integrated for DMSC IPC</t>
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr">
@@ -6740,7 +6749,7 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check in boot log, remote core should able to query of firmware is loaded or not </t>
+          <t xml:space="preserve">Confirm successful execution with DMSC firmware </t>
         </is>
       </c>
       <c r="L54" s="3" t="inlineStr">
@@ -6799,12 +6808,12 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1094</t>
+          <t>ETHFW-1097</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][IPC]IPC:Remote core invocation APIs for switch config should be stateless on remote core side</t>
+          <t>[EthFw][IPC]IPC: Support for remote core to query if switch R5 firmware has been loaded</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -6814,7 +6823,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1280,ETHFW-2172</t>
+          <t>ETHFW-1184,ETHFW-2172</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -6829,7 +6838,7 @@
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>IPC:Remote core invocation APIs for switch config should be stateless on remote core side</t>
+          <t>For generic kernel driver in mainline, dependency on pre-initialization is not good experience (people use different bootloader, boot sequence etc). So there should be a way to query of firmware is loaded and if not let driver load it from filesystem.</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
@@ -6839,7 +6848,7 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>client side application does not aware of state</t>
+          <t xml:space="preserve">Check in boot log, remote core should able to query of firmware is loaded or not </t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
@@ -6898,22 +6907,22 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1058</t>
+          <t>ETHFW-1094</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][IPC]IPC:Support for switch configuration from remote core</t>
+          <t>[EthFw][IPC]IPC:Remote core invocation APIs for switch config should be stateless on remote core side</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement,Requirement</t>
+          <t>Requirement,Requirement</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1168,ETHFW-2171,ETHFW-2172</t>
+          <t>ETHFW-1280,ETHFW-2172</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
@@ -6928,7 +6937,7 @@
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>IPC:Support for switch configuration from remote core</t>
+          <t>IPC:Remote core invocation APIs for switch config should be stateless on remote core side</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
@@ -6938,7 +6947,7 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Should able to configure Switch from all cores</t>
+          <t>client side application does not aware of state</t>
         </is>
       </c>
       <c r="L56" s="3" t="inlineStr">
@@ -6997,22 +7006,22 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1030</t>
+          <t>ETHFW-1058</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][IPC]IPC: Initial handshake and CPSW init completion notification</t>
+          <t>[EthFw][IPC]IPC:Support for switch configuration from remote core</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement</t>
+          <t>Requirement,Requirement,Requirement</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1245,ETHFW-2170</t>
+          <t>ETHFW-1168,ETHFW-2171,ETHFW-2172</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -7027,9 +7036,7 @@
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>IPC: Sync mechanism
-  Initial shared memory based handshake
-  Notification to remote cores on CPSW initial configuration completion</t>
+          <t>IPC:Support for switch configuration from remote core</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
@@ -7039,7 +7046,7 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">After successfully CPSW initialization, notification send to all remote cores </t>
+          <t>Should able to configure Switch from all cores</t>
         </is>
       </c>
       <c r="L57" s="3" t="inlineStr">
@@ -7098,22 +7105,22 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1025</t>
+          <t>ETHFW-1030</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][IPC]IPC: Integration with linux virtual driver running on A72 remote core</t>
+          <t>[EthFw][IPC]IPC: Initial handshake and CPSW init completion notification</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Requirement</t>
+          <t>Requirement,Requirement</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1143</t>
+          <t>ETHFW-1245,ETHFW-2170</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -7128,7 +7135,9 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware IPC should be integrated with linux virtual netdev driver running on A72 remote core</t>
+          <t>IPC: Sync mechanism
+  Initial shared memory based handshake
+  Notification to remote cores on CPSW initial configuration completion</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
@@ -7138,7 +7147,7 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Should able to run application successfully </t>
+          <t xml:space="preserve">After successfully CPSW initialization, notification send to all remote cores </t>
         </is>
       </c>
       <c r="L58" s="3" t="inlineStr">
@@ -7197,22 +7206,22 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1010</t>
+          <t>ETHFW-1025</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][IPC]IPC: All cores must allocate cores own MAC Address/IP address by sending msg to central IP/MAC resource manager running on master core</t>
+          <t>[EthFw][IPC]IPC: Integration with linux virtual driver running on A72 remote core</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1288,ETHFW-2172</t>
+          <t>ETHFW-1143</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -7227,7 +7236,7 @@
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>IPC: All cores must allocate cores own MAC Address/IP address by sending msg to central IP/MAC resource manager running on master core</t>
+          <t>Ethernet Firmware IPC should be integrated with linux virtual netdev driver running on A72 remote core</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
@@ -7237,7 +7246,7 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">All core must register them self by sending msg to master core </t>
+          <t xml:space="preserve">Should able to run application successfully </t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -7296,12 +7305,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-987</t>
+          <t>ETHFW-1010</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>[EthFw][IPC]IPC: Integration with CPSW LLD RTOS driver running on RTOS remote cores</t>
+          <t>[EthFw][IPC]IPC: All cores must allocate cores own MAC Address/IP address by sending msg to central IP/MAC resource manager running on master core</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
@@ -7311,7 +7320,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-1148,ETHFW-2171</t>
+          <t>ETHFW-1288,ETHFW-2172</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -7326,7 +7335,7 @@
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>Ethernet Firmware IPC should be integrated with Enet LLD RTOS driver running on RTOS remote cores.</t>
+          <t>IPC: All cores must allocate cores own MAC Address/IP address by sending msg to central IP/MAC resource manager running on master core</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
@@ -7336,7 +7345,7 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Should able to run application successfully </t>
+          <t xml:space="preserve">All core must register them self by sending msg to master core </t>
         </is>
       </c>
       <c r="L60" s="3" t="inlineStr">
@@ -7395,27 +7404,27 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2519</t>
+          <t>ETHFW-987</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Timestamped logs/traces</t>
+          <t>[EthFw][IPC]IPC: Integration with CPSW LLD RTOS driver running on RTOS remote cores</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Requirement</t>
+          <t>Requirement,Requirement</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2478</t>
+          <t>ETHFW-1148,ETHFW-2171</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>j721e-evm,j7200-evm,j784s4-evm</t>
+          <t>j721e-evm,j7200-evm</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
@@ -7425,38 +7434,17 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Verify that ETHFW tracing feature supports timestamping of logs/traces using an timestamp provider set by application.
-Reference timestamp provider:
-{code:c}
-#define SEC_TO_USEC (1000000ULL)
-static uint64_t EthApp_traceTs(void)
-{
-  static uint64_t ts = 0ULL;
-  TickType_t tickCnt;
-  uint64_t tickUsecs;
-  tickUsecs = SEC_TO_USEC / uint64_t)configTICK_RATE_HZ;
-  tickCnt = xTaskGetTickCount();
-  ts = (uint64_t)tickCnt * tickUsecs;
-  return ts;
-}
-/* Trace configuration */
-static EthFwTrace_Cfg gEthApp_traceCfg =
-{
-  .print        = appLogPrintf,
-  .traceTsFunc  = EthApp_traceTs,
-  .extTraceFunc = NULL,
-};
-EthFwTrace_init(&amp;gEthApp_traceCfg);{code}</t>
+          <t>Ethernet Firmware IPC should be integrated with Enet LLD RTOS driver running on RTOS remote cores.</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>J721E/J7200/J784S4 EVM.</t>
+          <t>J7 EVM with GESI Expansion card</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>ETHFW traces shall be printed with a timestamp.</t>
+          <t xml:space="preserve">Should able to run application successfully </t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
@@ -7515,12 +7503,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2524</t>
+          <t>ETHFW-2519</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Host port stats monitoring</t>
+          <t>EthFw: Timestamped logs/traces</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
@@ -7530,7 +7518,7 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2480</t>
+          <t>ETHFW-2478</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -7545,7 +7533,28 @@
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Verify that ETHFW is able to periodically monitor CPSW host port statistics and can notify ETHFW server application of such events.</t>
+          <t>Verify that ETHFW tracing feature supports timestamping of logs/traces using an timestamp provider set by application.
+Reference timestamp provider:
+{code:c}
+#define SEC_TO_USEC (1000000ULL)
+static uint64_t EthApp_traceTs(void)
+{
+  static uint64_t ts = 0ULL;
+  TickType_t tickCnt;
+  uint64_t tickUsecs;
+  tickUsecs = SEC_TO_USEC / uint64_t)configTICK_RATE_HZ;
+  tickCnt = xTaskGetTickCount();
+  ts = (uint64_t)tickCnt * tickUsecs;
+  return ts;
+}
+/* Trace configuration */
+static EthFwTrace_Cfg gEthApp_traceCfg =
+{
+  .print        = appLogPrintf,
+  .traceTsFunc  = EthApp_traceTs,
+  .extTraceFunc = NULL,
+};
+EthFwTrace_init(&amp;gEthApp_traceCfg);{code}</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
@@ -7555,7 +7564,7 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Host stats monitor callback should be called when a stats counter increase since previous periodic read.</t>
+          <t>ETHFW traces shall be printed with a timestamp.</t>
         </is>
       </c>
       <c r="L62" s="3" t="inlineStr">
@@ -7614,12 +7623,12 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2523</t>
+          <t>ETHFW-2524</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Ethernet port stats monitoring</t>
+          <t>EthFw: Host port stats monitoring</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
@@ -7629,7 +7638,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2479</t>
+          <t>ETHFW-2480</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -7644,7 +7653,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Verify that ETHFW is able to periodically monitor CPSW statistics and can notify ETHFW server application of such events.</t>
+          <t>Verify that ETHFW is able to periodically monitor CPSW host port statistics and can notify ETHFW server application of such events.</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
@@ -7654,7 +7663,7 @@
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Ethernet stats monitor callback should be called when a stats counter increase since previous periodic read.</t>
+          <t>Host stats monitor callback should be called when a stats counter increase since previous periodic read.</t>
         </is>
       </c>
       <c r="L63" s="3" t="inlineStr">
@@ -7713,12 +7722,12 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2522</t>
+          <t>ETHFW-2523</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Trace logging level (runtime)</t>
+          <t>EthFw: Ethernet port stats monitoring</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
@@ -7728,7 +7737,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2477</t>
+          <t>ETHFW-2479</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -7743,7 +7752,7 @@
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Verify ETHFW log levels can be set at runtime via EthFwTrace_setLevel().</t>
+          <t>Verify that ETHFW is able to periodically monitor CPSW statistics and can notify ETHFW server application of such events.</t>
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr">
@@ -7753,7 +7762,7 @@
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Log level shall be changed to the level selected by the application at runtime.</t>
+          <t>Ethernet stats monitor callback should be called when a stats counter increase since previous periodic read.</t>
         </is>
       </c>
       <c r="L64" s="3" t="inlineStr">
@@ -7812,12 +7821,12 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2521</t>
+          <t>ETHFW-2522</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Trace logging level (compile-time)</t>
+          <t>EthFw: Trace logging level (runtime)</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
@@ -7842,7 +7851,7 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Verify ETHFW log levels can be set at compile time via ETHFW_CFG_TRACE_LEVEL configuration parameter.</t>
+          <t>Verify ETHFW log levels can be set at runtime via EthFwTrace_setLevel().</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
@@ -7852,7 +7861,7 @@
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Build-time log level shall be set according to the build configuration parameter ETHFW_CFG_TRACE_LEVEL.</t>
+          <t>Log level shall be changed to the level selected by the application at runtime.</t>
         </is>
       </c>
       <c r="L65" s="3" t="inlineStr">
@@ -7911,12 +7920,12 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2520</t>
+          <t>ETHFW-2521</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>EthFw: Traces with unique error code</t>
+          <t>EthFw: Trace logging level (compile-time)</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
@@ -7926,7 +7935,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2489</t>
+          <t>ETHFW-2477</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -7941,21 +7950,7 @@
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>Verify that the external trace function gets called with a unique error code when ETHFW encounters an error condition at runtime.
-Reference unique error callback:
-{code:c}
-void EthApp_extTraceFunc(uint32_t errCode)
-{
-  appLogPrintf("Error code: %x\n", errCode);
-}
-/* Trace configuration */
-static EthFwTrace_Cfg gEthApp_traceCfg =
-{
-  .print        = appLogPrintf,
-  .traceTsFunc  = NULL,
-  .extTraceFunc = EthApp_extTraceFunc,
-};
-EthFwTrace_init(&amp;gEthApp_traceCfg); {code}</t>
+          <t>Verify ETHFW log levels can be set at compile time via ETHFW_CFG_TRACE_LEVEL configuration parameter.</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
@@ -7965,7 +7960,7 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>EthFw unique errors shall be logged using the provided callback function.</t>
+          <t>Build-time log level shall be set according to the build configuration parameter ETHFW_CFG_TRACE_LEVEL.</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
@@ -8014,32 +8009,32 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2526</t>
+          <t>ETHFW-2372</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>EthFw Reset Recovery Test Plan</t>
+          <t>ETHFW 9.x Release Test Plan (j7200)</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2515</t>
+          <t>ETHFW-2520</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>EthFw: FreeRTOS Reset Recovery test on EthFw standalone</t>
+          <t>EthFw: Traces with unique error code</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Requirement,Requirement,Requirement,Requirement,Requirement,Requirement</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2162,ETHFW-2160,ETHFW-2164,ETHFW-2163,ETHFW-2167,ETHFW-2161</t>
+          <t>ETHFW-2489</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -8054,18 +8049,31 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw.
-</t>
+          <t>Verify that the external trace function gets called with a unique error code when ETHFW encounters an error condition at runtime.
+Reference unique error callback:
+{code:c}
+void EthApp_extTraceFunc(uint32_t errCode)
+{
+  appLogPrintf("Error code: %x\n", errCode);
+}
+/* Trace configuration */
+static EthFwTrace_Cfg gEthApp_traceCfg =
+{
+  .print        = appLogPrintf,
+  .traceTsFunc  = NULL,
+  .extTraceFunc = EthApp_extTraceFunc,
+};
+EthFwTrace_init(&amp;gEthApp_traceCfg); {code}</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>J7 EVM with GESI Expansion card</t>
+          <t>J721E/J7200/J784S4 EVM.</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Recovery should be successful and post recovery packet transmission(ping/iperf should work)</t>
+          <t>EthFw unique errors shall be logged using the provided callback function.</t>
         </is>
       </c>
       <c r="L67" s="3" t="inlineStr">
@@ -8124,16 +8132,24 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2529</t>
+          <t>ETHFW-2515</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>EthFw: SafeRTOS Reset Recovery test on EthFw standalone</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr"/>
-      <c r="F68" s="3" t="inlineStr"/>
+          <t>EthFw: FreeRTOS Reset Recovery test on EthFw standalone</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Requirement,Requirement,Requirement,Requirement,Requirement,Requirement</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2162,ETHFW-2160,ETHFW-2164,ETHFW-2163,ETHFW-2167,ETHFW-2161</t>
+        </is>
+      </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
           <t>j721e-evm,j7200-evm,j784s4-evm</t>
@@ -8146,7 +8162,7 @@
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw.
+          <t xml:space="preserve">Test Reset recovery on EthFw.
 </t>
         </is>
       </c>
@@ -8216,12 +8232,12 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2528</t>
+          <t>ETHFW-2529</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>EthFw: SafeRTOS: Reset Recovery test on EthFw + MCAL Client</t>
+          <t>EthFw: SafeRTOS Reset Recovery test on EthFw standalone</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr"/>
@@ -8238,7 +8254,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw with MCAL client
+          <t xml:space="preserve">Test Reset recovery on EthFw.
 </t>
         </is>
       </c>
@@ -8308,12 +8324,12 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2527</t>
+          <t>ETHFW-2528</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>EthFw: FreeRTOS: Reset Recovery test on EthFw + MCAL Client</t>
+          <t>EthFw: SafeRTOS: Reset Recovery test on EthFw + MCAL Client</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr"/>
@@ -8330,7 +8346,7 @@
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw with MCAL client
+          <t xml:space="preserve">Test Reset recovery on EthFw with MCAL client
 </t>
         </is>
       </c>
@@ -8400,12 +8416,12 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2533</t>
+          <t>ETHFW-2527</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>EthFw: SafeRTOS: Reset Recovery test on EthFw + RTOS Client</t>
+          <t>EthFw: FreeRTOS: Reset Recovery test on EthFw + MCAL Client</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr"/>
@@ -8422,7 +8438,7 @@
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw with RTOS client
+          <t xml:space="preserve">Test Reset recovery on EthFw with MCAL client
 </t>
         </is>
       </c>
@@ -8492,12 +8508,12 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2532</t>
+          <t>ETHFW-2533</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>EthFw: FreeRTOS: Reset Recovery test on EthFw + RTOS Client</t>
+          <t>EthFw: SafeRTOS: Reset Recovery test on EthFw + RTOS Client</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr"/>
@@ -8514,7 +8530,7 @@
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw with RTOS client
+          <t xml:space="preserve">Test Reset recovery on EthFw with RTOS client
 </t>
         </is>
       </c>
@@ -8584,12 +8600,12 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2531</t>
+          <t>ETHFW-2532</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>EthFw: FreeRTOS: Reset Recovery test on EthFw + Linux Client</t>
+          <t>EthFw: FreeRTOS: Reset Recovery test on EthFw + RTOS Client</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr"/>
@@ -8606,7 +8622,7 @@
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw with Linux client
+          <t xml:space="preserve">Test Reset recovery on EthFw with RTOS client
 </t>
         </is>
       </c>
@@ -8676,12 +8692,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2530</t>
+          <t>ETHFW-2531</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>EthFw: SafeRTOS: Reset Recovery test on EthFw + Linux Client</t>
+          <t>EthFw: FreeRTOS: Reset Recovery test on EthFw + Linux Client</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr"/>
@@ -8698,7 +8714,7 @@
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw with Linux client
+          <t xml:space="preserve">Test Reset recovery on EthFw with Linux client
 </t>
         </is>
       </c>
@@ -8768,12 +8784,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2534</t>
+          <t>ETHFW-2530</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>EthFw: FreeRTOS Reset Recovery Robust test</t>
+          <t>EthFw: SafeRTOS: Reset Recovery test on EthFw + Linux Client</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr"/>
@@ -8790,7 +8806,7 @@
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw by triggering multiple iterations of recovery
+          <t xml:space="preserve">Test Reset recovery on EthFw with Linux client
 </t>
         </is>
       </c>
@@ -8860,12 +8876,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2535</t>
+          <t>ETHFW-2534</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>EthFw: SafeRTOS Reset Recovery Robust test</t>
+          <t>EthFw: FreeRTOS Reset Recovery Robust test</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr"/>
@@ -8882,7 +8898,7 @@
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test Reset recovery on EthFw by triggering multiple iterations of recovery
+          <t xml:space="preserve">Test Reset recovery on EthFw by triggering multiple iterations of recovery
 </t>
         </is>
       </c>
@@ -8939,9 +8955,101 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2526</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>EthFw Reset Recovery Test Plan</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2535</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>EthFw: SafeRTOS Reset Recovery Robust test</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr"/>
+      <c r="F77" s="3" t="inlineStr"/>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>j721e-evm,j7200-evm,j784s4-evm</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test Reset recovery on EthFw by triggering multiple iterations of recovery
+</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>J7 EVM with GESI Expansion card</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>Recovery should be successful and post recovery packet transmission(ping/iperf should work)</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
+        <is>
+          <t>Requirements-Analysis</t>
+        </is>
+      </c>
+      <c r="N77" s="3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="O77" s="3" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="P77" s="3" t="inlineStr">
+        <is>
+          <t>EthFw</t>
+        </is>
+      </c>
+      <c r="Q77" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2506</t>
+        </is>
+      </c>
+      <c r="R77" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW 9.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S77" s="3" t="inlineStr"/>
+      <c r="T77" s="3" t="inlineStr"/>
+      <c r="U77" s="9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U76"/>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <autoFilter ref="A1:U77"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -8954,11 +9062,11 @@
   <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="16"/>
-    <col customWidth="1" max="2" min="2" width="23"/>
-    <col customWidth="1" max="3" min="3" width="67"/>
-    <col customWidth="1" max="4" min="4" width="30"/>
-    <col customWidth="1" max="5" min="5" width="30"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="67" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9901,14 +10009,14 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A35:A42"/>
+    <mergeCell ref="B13:B23"/>
+    <mergeCell ref="B24:B28"/>
+    <mergeCell ref="B38:B42"/>
     <mergeCell ref="A2:A34"/>
-    <mergeCell ref="A35:A42"/>
-    <mergeCell ref="B38:B42"/>
     <mergeCell ref="B30:B33"/>
-    <mergeCell ref="B24:B28"/>
-    <mergeCell ref="B13:B23"/>
   </mergeCells>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -9921,10 +10029,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="12"/>
-    <col customWidth="1" max="2" min="2" width="12"/>
-    <col customWidth="1" max="3" min="3" width="12"/>
-    <col customWidth="1" max="4" min="4" width="100"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10148,6 +10256,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ethfw: release_reports: Update test, bi-di and SA reports for SDK 10.1
- Update SDK 10.1 test reports.
- Update Static Analysis report for EthFw.
- Update bi-directional traceability report for EthFw.

Fixes: ETHFW-2983

Signed-off-by: Sonu Alam <s-alam@ti.com>
</commit_message>
<xml_diff>
--- a/docs/test_report/ethfw_testreport_j7200.xlsx
+++ b/docs/test_report/ethfw_testreport_j7200.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="4" name="_xlnm._FilterDatabase">'Test Strategy Compliance'!$A$1:$E$5</definedName>
-    <definedName hidden="1" localSheetId="5" name="_xlnm._FilterDatabase">'Test Plan | Execution Report'!$A$1:$U$181</definedName>
+    <definedName hidden="1" localSheetId="5" name="_xlnm._FilterDatabase">'Test Plan | Execution Report'!$A$1:$U$186</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -724,7 +724,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2024-08-07 04:16:53.028009-05:00 CDT</t>
+          <t>2024-11-25 04:40:39.408674-06:00 CDT</t>
         </is>
       </c>
     </row>
@@ -811,12 +811,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>76</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -922,12 +922,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>100</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -1033,12 +1033,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>181</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>185</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1124,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -1220,12 +1220,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="inlineStr">
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4">
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="7" t="inlineStr">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -1434,7 +1434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U181"/>
+  <dimension ref="A1:U186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="17"/>
@@ -1652,12 +1652,12 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr"/>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr"/>
@@ -1855,12 +1855,12 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr"/>
@@ -1956,12 +1956,12 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr"/>
@@ -2057,12 +2057,12 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr"/>
@@ -2158,12 +2158,12 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr"/>
@@ -2259,12 +2259,12 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr"/>
@@ -2360,12 +2360,12 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr"/>
@@ -2461,12 +2461,12 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr"/>
@@ -2562,12 +2562,12 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S11" s="3" t="inlineStr"/>
@@ -2663,12 +2663,12 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S12" s="3" t="inlineStr"/>
@@ -2764,12 +2764,12 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R13" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S13" s="3" t="inlineStr"/>
@@ -2866,12 +2866,12 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S14" s="3" t="inlineStr"/>
@@ -2966,24 +2966,16 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
-        </is>
-      </c>
-      <c r="S15" s="3" t="inlineStr">
-        <is>
-          <t>ETHFW-2838</t>
-        </is>
-      </c>
-      <c r="T15" s="3" t="inlineStr">
-        <is>
-          <t>ETHFW: Linux: Virtual MAC port doesn't return error when entering promisc mode</t>
-        </is>
-      </c>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr"/>
+      <c r="T15" s="3" t="inlineStr"/>
       <c r="U15" s="11" t="inlineStr">
         <is>
           <t>Fail</t>
@@ -3075,12 +3067,12 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S16" s="3" t="inlineStr"/>
@@ -3176,12 +3168,12 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S17" s="3" t="inlineStr"/>
@@ -3277,12 +3269,12 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S18" s="3" t="inlineStr"/>
@@ -3379,12 +3371,12 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S19" s="3" t="inlineStr"/>
@@ -3480,12 +3472,12 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr"/>
@@ -3580,12 +3572,12 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S21" s="3" t="inlineStr"/>
@@ -3683,12 +3675,12 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S22" s="3" t="inlineStr"/>
@@ -3785,12 +3777,12 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S23" s="3" t="inlineStr"/>
@@ -3884,12 +3876,12 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr"/>
@@ -3983,12 +3975,12 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr"/>
@@ -4082,12 +4074,12 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr"/>
@@ -4181,12 +4173,12 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr"/>
@@ -4280,12 +4272,12 @@
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R28" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S28" s="3" t="inlineStr"/>
@@ -4380,12 +4372,12 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R29" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S29" s="3" t="inlineStr"/>
@@ -4479,12 +4471,12 @@
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr"/>
@@ -4578,12 +4570,12 @@
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S31" s="3" t="inlineStr"/>
@@ -4694,12 +4686,12 @@
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R32" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S32" s="3" t="inlineStr"/>
@@ -4812,12 +4804,12 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R33" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S33" s="3" t="inlineStr"/>
@@ -4914,12 +4906,12 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R34" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S34" s="3" t="inlineStr"/>
@@ -5007,12 +4999,12 @@
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R35" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S35" s="3" t="inlineStr"/>
@@ -5099,12 +5091,12 @@
       </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R36" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S36" s="3" t="inlineStr"/>
@@ -5215,12 +5207,12 @@
       </c>
       <c r="Q37" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R37" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S37" s="3" t="inlineStr"/>
@@ -5331,12 +5323,12 @@
       </c>
       <c r="Q38" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R38" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S38" s="3" t="inlineStr"/>
@@ -5431,12 +5423,12 @@
       </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R39" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S39" s="3" t="inlineStr"/>
@@ -5523,12 +5515,12 @@
       </c>
       <c r="Q40" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R40" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S40" s="3" t="inlineStr"/>
@@ -5615,12 +5607,12 @@
       </c>
       <c r="Q41" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R41" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S41" s="3" t="inlineStr"/>
@@ -5707,12 +5699,12 @@
       </c>
       <c r="Q42" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R42" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S42" s="3" t="inlineStr"/>
@@ -5799,19 +5791,27 @@
       </c>
       <c r="Q43" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R43" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
-        </is>
-      </c>
-      <c r="S43" s="3" t="inlineStr"/>
-      <c r="T43" s="3" t="inlineStr"/>
-      <c r="U43" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S43" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2974</t>
+        </is>
+      </c>
+      <c r="T43" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW: RTOS: Reset recovery fails with RTOS client</t>
+        </is>
+      </c>
+      <c r="U43" s="11" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>
@@ -5891,12 +5891,12 @@
       </c>
       <c r="Q44" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R44" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S44" s="3" t="inlineStr"/>
@@ -5984,12 +5984,12 @@
       </c>
       <c r="Q45" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R45" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S45" s="3" t="inlineStr"/>
@@ -6078,12 +6078,12 @@
       </c>
       <c r="Q46" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R46" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S46" s="3" t="inlineStr"/>
@@ -6170,12 +6170,12 @@
       </c>
       <c r="Q47" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R47" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S47" s="3" t="inlineStr"/>
@@ -6262,12 +6262,12 @@
       </c>
       <c r="Q48" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R48" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S48" s="3" t="inlineStr"/>
@@ -6368,19 +6368,19 @@
       </c>
       <c r="Q49" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R49" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S49" s="3" t="inlineStr"/>
       <c r="T49" s="3" t="inlineStr"/>
-      <c r="U49" s="11" t="inlineStr">
-        <is>
-          <t>Fail</t>
+      <c r="U49" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6473,12 +6473,12 @@
       </c>
       <c r="Q50" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R50" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S50" s="3" t="inlineStr"/>
@@ -6579,12 +6579,12 @@
       </c>
       <c r="Q51" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R51" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S51" s="3" t="inlineStr"/>
@@ -6684,12 +6684,12 @@
       </c>
       <c r="Q52" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R52" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S52" s="3" t="inlineStr"/>
@@ -6788,19 +6788,19 @@
       </c>
       <c r="Q53" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R53" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S53" s="3" t="inlineStr"/>
       <c r="T53" s="3" t="inlineStr"/>
-      <c r="U53" s="11" t="inlineStr">
-        <is>
-          <t>Fail</t>
+      <c r="U53" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6892,12 +6892,12 @@
       </c>
       <c r="Q54" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R54" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S54" s="3" t="inlineStr"/>
@@ -6996,12 +6996,12 @@
       </c>
       <c r="Q55" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R55" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S55" s="3" t="inlineStr"/>
@@ -7101,12 +7101,12 @@
       </c>
       <c r="Q56" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R56" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S56" s="3" t="inlineStr"/>
@@ -7207,12 +7207,12 @@
       </c>
       <c r="Q57" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R57" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S57" s="3" t="inlineStr"/>
@@ -7312,12 +7312,12 @@
       </c>
       <c r="Q58" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R58" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S58" s="3" t="inlineStr"/>
@@ -7416,12 +7416,12 @@
       </c>
       <c r="Q59" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R59" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S59" s="3" t="inlineStr"/>
@@ -7522,12 +7522,12 @@
       </c>
       <c r="Q60" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R60" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S60" s="3" t="inlineStr"/>
@@ -7621,12 +7621,12 @@
       </c>
       <c r="Q61" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R61" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S61" s="3" t="inlineStr"/>
@@ -7727,12 +7727,12 @@
       </c>
       <c r="Q62" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R62" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S62" s="3" t="inlineStr"/>
@@ -7829,12 +7829,12 @@
       </c>
       <c r="Q63" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R63" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S63" s="3" t="inlineStr"/>
@@ -7937,12 +7937,12 @@
       </c>
       <c r="Q64" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R64" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S64" s="3" t="inlineStr"/>
@@ -8045,12 +8045,12 @@
       </c>
       <c r="Q65" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R65" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S65" s="3" t="inlineStr"/>
@@ -8146,12 +8146,12 @@
       </c>
       <c r="Q66" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R66" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S66" s="3" t="inlineStr"/>
@@ -8249,12 +8249,12 @@
       </c>
       <c r="Q67" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R67" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S67" s="3" t="inlineStr"/>
@@ -8354,12 +8354,12 @@
       </c>
       <c r="Q68" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R68" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S68" s="3" t="inlineStr"/>
@@ -8453,12 +8453,12 @@
       </c>
       <c r="Q69" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R69" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S69" s="3" t="inlineStr"/>
@@ -8555,12 +8555,12 @@
       </c>
       <c r="Q70" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R70" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S70" s="3" t="inlineStr"/>
@@ -8658,12 +8658,12 @@
       </c>
       <c r="Q71" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R71" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S71" s="3" t="inlineStr"/>
@@ -8769,12 +8769,12 @@
       </c>
       <c r="Q72" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R72" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S72" s="3" t="inlineStr"/>
@@ -8868,12 +8868,12 @@
       </c>
       <c r="Q73" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R73" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S73" s="3" t="inlineStr"/>
@@ -8967,12 +8967,12 @@
       </c>
       <c r="Q74" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R74" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S74" s="3" t="inlineStr"/>
@@ -9066,12 +9066,12 @@
       </c>
       <c r="Q75" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R75" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S75" s="3" t="inlineStr"/>
@@ -9165,12 +9165,12 @@
       </c>
       <c r="Q76" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R76" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S76" s="3" t="inlineStr"/>
@@ -9268,12 +9268,12 @@
       </c>
       <c r="Q77" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R77" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S77" s="3" t="inlineStr"/>
@@ -9367,12 +9367,12 @@
       </c>
       <c r="Q78" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R78" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S78" s="3" t="inlineStr"/>
@@ -9466,12 +9466,12 @@
       </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R79" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S79" s="3" t="inlineStr"/>
@@ -9565,12 +9565,12 @@
       </c>
       <c r="Q80" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R80" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S80" s="3" t="inlineStr"/>
@@ -9664,12 +9664,12 @@
       </c>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R81" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S81" s="3" t="inlineStr"/>
@@ -9763,12 +9763,12 @@
       </c>
       <c r="Q82" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R82" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S82" s="3" t="inlineStr"/>
@@ -9862,12 +9862,12 @@
       </c>
       <c r="Q83" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R83" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S83" s="3" t="inlineStr"/>
@@ -9963,12 +9963,12 @@
       </c>
       <c r="Q84" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R84" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S84" s="3" t="inlineStr"/>
@@ -10062,12 +10062,12 @@
       </c>
       <c r="Q85" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R85" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S85" s="3" t="inlineStr"/>
@@ -10161,12 +10161,12 @@
       </c>
       <c r="Q86" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R86" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S86" s="3" t="inlineStr"/>
@@ -10260,12 +10260,12 @@
       </c>
       <c r="Q87" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R87" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S87" s="3" t="inlineStr"/>
@@ -10380,12 +10380,12 @@
       </c>
       <c r="Q88" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R88" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S88" s="3" t="inlineStr"/>
@@ -10479,12 +10479,12 @@
       </c>
       <c r="Q89" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R89" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S89" s="3" t="inlineStr"/>
@@ -10578,12 +10578,12 @@
       </c>
       <c r="Q90" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R90" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S90" s="3" t="inlineStr"/>
@@ -10677,12 +10677,12 @@
       </c>
       <c r="Q91" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R91" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S91" s="3" t="inlineStr"/>
@@ -10776,12 +10776,12 @@
       </c>
       <c r="Q92" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R92" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S92" s="3" t="inlineStr"/>
@@ -10889,12 +10889,12 @@
       </c>
       <c r="Q93" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R93" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S93" s="3" t="inlineStr"/>
@@ -10992,12 +10992,12 @@
       </c>
       <c r="Q94" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R94" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S94" s="3" t="inlineStr"/>
@@ -11098,12 +11098,12 @@
       </c>
       <c r="Q95" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R95" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S95" s="3" t="inlineStr"/>
@@ -11204,12 +11204,12 @@
       </c>
       <c r="Q96" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R96" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S96" s="3" t="inlineStr"/>
@@ -11306,12 +11306,12 @@
       </c>
       <c r="Q97" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R97" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S97" s="3" t="inlineStr"/>
@@ -11407,12 +11407,12 @@
       </c>
       <c r="Q98" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R98" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S98" s="3" t="inlineStr"/>
@@ -11510,12 +11510,12 @@
       </c>
       <c r="Q99" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R99" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S99" s="3" t="inlineStr"/>
@@ -11613,12 +11613,12 @@
       </c>
       <c r="Q100" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R100" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S100" s="3" t="inlineStr"/>
@@ -11717,12 +11717,12 @@
       </c>
       <c r="Q101" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R101" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S101" s="3" t="inlineStr"/>
@@ -11820,12 +11820,12 @@
       </c>
       <c r="Q102" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R102" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S102" s="3" t="inlineStr"/>
@@ -11921,24 +11921,16 @@
       </c>
       <c r="Q103" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R103" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
-        </is>
-      </c>
-      <c r="S103" s="3" t="inlineStr">
-        <is>
-          <t>ETHFW-2575</t>
-        </is>
-      </c>
-      <c r="T103" s="3" t="inlineStr">
-        <is>
-          <t>CPSW error flags are not getting updated in UDMA host packet descriptor</t>
-        </is>
-      </c>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S103" s="3" t="inlineStr"/>
+      <c r="T103" s="3" t="inlineStr"/>
       <c r="U103" s="11" t="inlineStr">
         <is>
           <t>Fail</t>
@@ -12031,12 +12023,12 @@
       </c>
       <c r="Q104" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R104" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S104" s="3" t="inlineStr"/>
@@ -12133,12 +12125,12 @@
       </c>
       <c r="Q105" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R105" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S105" s="3" t="inlineStr"/>
@@ -12235,12 +12227,12 @@
       </c>
       <c r="Q106" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R106" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S106" s="3" t="inlineStr"/>
@@ -12337,12 +12329,12 @@
       </c>
       <c r="Q107" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R107" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S107" s="3" t="inlineStr"/>
@@ -12439,12 +12431,12 @@
       </c>
       <c r="Q108" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R108" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S108" s="3" t="inlineStr"/>
@@ -12541,12 +12533,12 @@
       </c>
       <c r="Q109" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R109" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S109" s="3" t="inlineStr"/>
@@ -12643,12 +12635,12 @@
       </c>
       <c r="Q110" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R110" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S110" s="3" t="inlineStr"/>
@@ -12745,12 +12737,12 @@
       </c>
       <c r="Q111" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R111" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S111" s="3" t="inlineStr"/>
@@ -12847,12 +12839,12 @@
       </c>
       <c r="Q112" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R112" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S112" s="3" t="inlineStr"/>
@@ -12949,12 +12941,12 @@
       </c>
       <c r="Q113" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R113" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S113" s="3" t="inlineStr"/>
@@ -13051,12 +13043,12 @@
       </c>
       <c r="Q114" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R114" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S114" s="3" t="inlineStr"/>
@@ -13153,12 +13145,12 @@
       </c>
       <c r="Q115" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R115" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S115" s="3" t="inlineStr"/>
@@ -13255,12 +13247,12 @@
       </c>
       <c r="Q116" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R116" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S116" s="3" t="inlineStr"/>
@@ -13357,12 +13349,12 @@
       </c>
       <c r="Q117" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R117" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S117" s="3" t="inlineStr"/>
@@ -13459,12 +13451,12 @@
       </c>
       <c r="Q118" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R118" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S118" s="3" t="inlineStr"/>
@@ -13561,12 +13553,12 @@
       </c>
       <c r="Q119" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R119" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S119" s="3" t="inlineStr"/>
@@ -13663,12 +13655,12 @@
       </c>
       <c r="Q120" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R120" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S120" s="3" t="inlineStr"/>
@@ -13765,12 +13757,12 @@
       </c>
       <c r="Q121" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R121" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S121" s="3" t="inlineStr"/>
@@ -13867,12 +13859,12 @@
       </c>
       <c r="Q122" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R122" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S122" s="3" t="inlineStr"/>
@@ -13969,12 +13961,12 @@
       </c>
       <c r="Q123" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R123" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S123" s="3" t="inlineStr"/>
@@ -14071,12 +14063,12 @@
       </c>
       <c r="Q124" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R124" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S124" s="3" t="inlineStr"/>
@@ -14173,12 +14165,12 @@
       </c>
       <c r="Q125" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R125" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S125" s="3" t="inlineStr"/>
@@ -14275,12 +14267,12 @@
       </c>
       <c r="Q126" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R126" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S126" s="3" t="inlineStr"/>
@@ -14377,12 +14369,12 @@
       </c>
       <c r="Q127" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R127" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S127" s="3" t="inlineStr"/>
@@ -14479,12 +14471,12 @@
       </c>
       <c r="Q128" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R128" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S128" s="3" t="inlineStr"/>
@@ -14581,12 +14573,12 @@
       </c>
       <c r="Q129" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R129" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S129" s="3" t="inlineStr"/>
@@ -14683,12 +14675,12 @@
       </c>
       <c r="Q130" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R130" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S130" s="3" t="inlineStr"/>
@@ -14785,12 +14777,12 @@
       </c>
       <c r="Q131" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R131" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S131" s="3" t="inlineStr"/>
@@ -14887,12 +14879,12 @@
       </c>
       <c r="Q132" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R132" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S132" s="3" t="inlineStr"/>
@@ -14989,12 +14981,12 @@
       </c>
       <c r="Q133" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R133" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S133" s="3" t="inlineStr"/>
@@ -15091,12 +15083,12 @@
       </c>
       <c r="Q134" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R134" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S134" s="3" t="inlineStr"/>
@@ -15193,12 +15185,12 @@
       </c>
       <c r="Q135" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R135" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S135" s="3" t="inlineStr"/>
@@ -15295,12 +15287,12 @@
       </c>
       <c r="Q136" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R136" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S136" s="3" t="inlineStr"/>
@@ -15397,12 +15389,12 @@
       </c>
       <c r="Q137" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R137" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S137" s="3" t="inlineStr"/>
@@ -15499,12 +15491,12 @@
       </c>
       <c r="Q138" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R138" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S138" s="3" t="inlineStr"/>
@@ -15601,12 +15593,12 @@
       </c>
       <c r="Q139" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R139" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S139" s="3" t="inlineStr"/>
@@ -15703,12 +15695,12 @@
       </c>
       <c r="Q140" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R140" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S140" s="3" t="inlineStr"/>
@@ -15805,12 +15797,12 @@
       </c>
       <c r="Q141" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R141" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S141" s="3" t="inlineStr"/>
@@ -15907,12 +15899,12 @@
       </c>
       <c r="Q142" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R142" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S142" s="3" t="inlineStr"/>
@@ -16009,12 +16001,12 @@
       </c>
       <c r="Q143" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R143" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S143" s="3" t="inlineStr"/>
@@ -16111,12 +16103,12 @@
       </c>
       <c r="Q144" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R144" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S144" s="3" t="inlineStr"/>
@@ -16213,12 +16205,12 @@
       </c>
       <c r="Q145" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R145" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S145" s="3" t="inlineStr"/>
@@ -16315,12 +16307,12 @@
       </c>
       <c r="Q146" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R146" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S146" s="3" t="inlineStr"/>
@@ -16417,12 +16409,12 @@
       </c>
       <c r="Q147" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R147" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S147" s="3" t="inlineStr"/>
@@ -16519,12 +16511,12 @@
       </c>
       <c r="Q148" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R148" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S148" s="3" t="inlineStr"/>
@@ -16621,12 +16613,12 @@
       </c>
       <c r="Q149" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R149" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S149" s="3" t="inlineStr"/>
@@ -16723,12 +16715,12 @@
       </c>
       <c r="Q150" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R150" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S150" s="3" t="inlineStr"/>
@@ -16825,12 +16817,12 @@
       </c>
       <c r="Q151" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R151" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S151" s="3" t="inlineStr"/>
@@ -16927,12 +16919,12 @@
       </c>
       <c r="Q152" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R152" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S152" s="3" t="inlineStr"/>
@@ -17029,12 +17021,12 @@
       </c>
       <c r="Q153" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R153" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S153" s="3" t="inlineStr"/>
@@ -17131,12 +17123,12 @@
       </c>
       <c r="Q154" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R154" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S154" s="3" t="inlineStr"/>
@@ -17233,12 +17225,12 @@
       </c>
       <c r="Q155" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R155" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S155" s="3" t="inlineStr"/>
@@ -17335,12 +17327,12 @@
       </c>
       <c r="Q156" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R156" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S156" s="3" t="inlineStr"/>
@@ -17437,12 +17429,12 @@
       </c>
       <c r="Q157" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R157" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S157" s="3" t="inlineStr"/>
@@ -17539,12 +17531,12 @@
       </c>
       <c r="Q158" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R158" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S158" s="3" t="inlineStr"/>
@@ -17641,12 +17633,12 @@
       </c>
       <c r="Q159" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R159" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S159" s="3" t="inlineStr"/>
@@ -17743,12 +17735,12 @@
       </c>
       <c r="Q160" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R160" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S160" s="3" t="inlineStr"/>
@@ -17845,12 +17837,12 @@
       </c>
       <c r="Q161" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R161" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S161" s="3" t="inlineStr"/>
@@ -17947,12 +17939,12 @@
       </c>
       <c r="Q162" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R162" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S162" s="3" t="inlineStr"/>
@@ -18049,12 +18041,12 @@
       </c>
       <c r="Q163" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R163" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S163" s="3" t="inlineStr"/>
@@ -18151,12 +18143,12 @@
       </c>
       <c r="Q164" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R164" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S164" s="3" t="inlineStr"/>
@@ -18253,12 +18245,12 @@
       </c>
       <c r="Q165" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R165" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S165" s="3" t="inlineStr"/>
@@ -18355,12 +18347,12 @@
       </c>
       <c r="Q166" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R166" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S166" s="3" t="inlineStr"/>
@@ -18457,12 +18449,12 @@
       </c>
       <c r="Q167" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R167" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S167" s="3" t="inlineStr"/>
@@ -18559,12 +18551,12 @@
       </c>
       <c r="Q168" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R168" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S168" s="3" t="inlineStr"/>
@@ -18661,12 +18653,12 @@
       </c>
       <c r="Q169" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R169" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S169" s="3" t="inlineStr"/>
@@ -18763,12 +18755,12 @@
       </c>
       <c r="Q170" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R170" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S170" s="3" t="inlineStr"/>
@@ -18865,12 +18857,12 @@
       </c>
       <c r="Q171" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R171" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S171" s="3" t="inlineStr"/>
@@ -18967,12 +18959,12 @@
       </c>
       <c r="Q172" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R172" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S172" s="3" t="inlineStr"/>
@@ -19069,12 +19061,12 @@
       </c>
       <c r="Q173" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R173" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S173" s="3" t="inlineStr"/>
@@ -19171,12 +19163,12 @@
       </c>
       <c r="Q174" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R174" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S174" s="3" t="inlineStr"/>
@@ -19273,12 +19265,12 @@
       </c>
       <c r="Q175" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R175" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S175" s="3" t="inlineStr"/>
@@ -19375,12 +19367,12 @@
       </c>
       <c r="Q176" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R176" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S176" s="3" t="inlineStr"/>
@@ -19477,12 +19469,12 @@
       </c>
       <c r="Q177" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R177" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S177" s="3" t="inlineStr"/>
@@ -19579,12 +19571,12 @@
       </c>
       <c r="Q178" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R178" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S178" s="3" t="inlineStr"/>
@@ -19681,12 +19673,12 @@
       </c>
       <c r="Q179" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R179" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S179" s="3" t="inlineStr"/>
@@ -19783,12 +19775,12 @@
       </c>
       <c r="Q180" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R180" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S180" s="3" t="inlineStr"/>
@@ -19885,12 +19877,12 @@
       </c>
       <c r="Q181" s="3" t="inlineStr">
         <is>
-          <t>ETHFW-2828</t>
+          <t>ETHFW-2970</t>
         </is>
       </c>
       <c r="R181" s="3" t="inlineStr">
         <is>
-          <t>ETHFW 10.0 Release Test Run (j7200)</t>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
         </is>
       </c>
       <c r="S181" s="3" t="inlineStr"/>
@@ -19901,8 +19893,534 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2971</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW VLAN test plan</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2892</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>Shared multicast test with VLAN</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>Requirement,Requirement</t>
+        </is>
+      </c>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2895,ETHFW-2891</t>
+        </is>
+      </c>
+      <c r="G182" s="3" t="inlineStr">
+        <is>
+          <t>j784s4-evm</t>
+        </is>
+      </c>
+      <c r="H182" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="I182" s="3" t="inlineStr">
+        <is>
+          <t>Shared multicast is a traffic that is supposed to be reached to multiple clients post registration.
+This test exercises the same with and without VLAN.
+As we lwip bridge does not support VLAN, shared multicast should reach all the clients who have reigstered with that multicast address irrespective of VLAN in NON-VEPA case.
+Similarly shared multicast should reach only to the specific client who have registered with that multicast address with VLAN. As we are honoring VLAN with shared multicast on devices where VEPA is enabled.</t>
+        </is>
+      </c>
+      <c r="J182" s="3" t="inlineStr">
+        <is>
+          <t>1. Join VLAN from client1 and another VLAN from client2 (do vlan_join from Linux client or add an instruction in RTOS client)
+2. Register to same shared multicast address from client1 and client2 but with different VLANs.
+3. Send a packet with dst mac as shared multicast address with different combinations (i.e. with VLAN 0, client1's VLAN, client2's VLAN and unknown VLAN).
+3. Check packet receive at clients. See the success criteria for details.</t>
+        </is>
+      </c>
+      <c r="K182" s="3" t="inlineStr">
+        <is>
+          <t>Shared multicast should reach all the clients who have reigstered with that multicast address irrespective of VLAN in NON-VEPA case.
+Shared multicast should reach only to the specific client who have registered with that multicast address with VLAN. As we are honoring VLAN with shared multicast on devices where VEPA is enabled.</t>
+        </is>
+      </c>
+      <c r="L182" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M182" s="3" t="inlineStr">
+        <is>
+          <t>Requirements-Analysis</t>
+        </is>
+      </c>
+      <c r="N182" s="3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="O182" s="3" t="inlineStr">
+        <is>
+          <t>Sanity</t>
+        </is>
+      </c>
+      <c r="P182" s="3" t="inlineStr">
+        <is>
+          <t>EthFw</t>
+        </is>
+      </c>
+      <c r="Q182" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2970</t>
+        </is>
+      </c>
+      <c r="R182" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S182" s="3" t="inlineStr"/>
+      <c r="T182" s="3" t="inlineStr"/>
+      <c r="U182" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2971</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW VLAN test plan</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2876</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>VLANs honored with unicast packets with multiple clients</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="F183" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2895</t>
+        </is>
+      </c>
+      <c r="G183" s="3" t="inlineStr">
+        <is>
+          <t>j721e-evm,j7200-evm,j784s4-evm</t>
+        </is>
+      </c>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="I183" s="3" t="inlineStr">
+        <is>
+          <t>VLAN tagged unicast packets should only be reached to the client if the client has joined that VLAN or if any other client has joined that VLAN else should be dropped.
+When multiple clients join different VLAN and we send a packet of 1 client's mac address say M1 with another client's VLAN say V2, then still packet is being received by M1 client. This has been taken as a known limitation so that we use less number of ALE and Classifier entires out of box. Note that not all VLAN packets will be received by M1. VLAN packets who's unicast address is M1 and VLAN registered by M1 or any other client will be received by M1. Unknown VLAN tagged packets with source mac address as M1 will still not be received by M1. This has been ensured excluding host port from unknown VLAN member list mask.</t>
+        </is>
+      </c>
+      <c r="J183" s="3" t="inlineStr">
+        <is>
+          <t>1. Join VLAN 1024 from client C1, and VLAN 1025 from client C2. (do vlan_join from Linux client or add an instruction in RTOS client)
+2. Send unicast packets of C1's MAC address but with VLAN 1025 (C2's VLAN) (use packETH)
+3. Check packet receive at client, and observe that packet should reach to any client (due to known limitation)
+4. Make sure you test the reverse and C1 with 1024 and C2 with 1025 vlan as well (i.e. correct VLAN)
+5. Send an uknown VLAN (say 102) with C1's mac address. Packet should NOT be reached to C1. Do that same with C2 as well.
+6. Packets with only registered VLAN should be propagated to host port, that too post any client joins that VLAN.</t>
+        </is>
+      </c>
+      <c r="K183" s="3" t="inlineStr">
+        <is>
+          <t>Check packet receive at client, and observe that packet should NOT reach to any client</t>
+        </is>
+      </c>
+      <c r="L183" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M183" s="3" t="inlineStr">
+        <is>
+          <t>Requirements-Analysis</t>
+        </is>
+      </c>
+      <c r="N183" s="3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="O183" s="3" t="inlineStr">
+        <is>
+          <t>Sanity</t>
+        </is>
+      </c>
+      <c r="P183" s="3" t="inlineStr">
+        <is>
+          <t>EthFw</t>
+        </is>
+      </c>
+      <c r="Q183" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2970</t>
+        </is>
+      </c>
+      <c r="R183" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S183" s="3" t="inlineStr"/>
+      <c r="T183" s="3" t="inlineStr"/>
+      <c r="U183" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2971</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW VLAN test plan</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2875</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>VLAN Broadcast packets duplicated to clients in VEPA</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="F184" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2895</t>
+        </is>
+      </c>
+      <c r="G184" s="3" t="inlineStr">
+        <is>
+          <t>j784s4-evm</t>
+        </is>
+      </c>
+      <c r="H184" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="I184" s="3" t="inlineStr">
+        <is>
+          <t>VLAN Broadcast packets should only be duplicated to clients who have joined that VLAN. This functionality should work with VEPA on J784S4.</t>
+        </is>
+      </c>
+      <c r="J184" s="3" t="inlineStr">
+        <is>
+          <t>1. Join VLAN from client (do vlan_join from Linux client or add an instruction in RTOS client)
+2. Send a Broadcast + VLAN of above joined packet to any of switch Port (use packETH)
+3. Check packet receive at client, and observe that packet should reach to clients
+4. Make sure that other external ports which are not part of that VLAN should not receive those packets (use wireshark to track that)</t>
+        </is>
+      </c>
+      <c r="K184" s="3" t="inlineStr">
+        <is>
+          <t>Check packet receive at client, and observe that packet should reach to clients
+Make sure that other external ports which are not part of that VLAN should not receive those packets (use wireshark to track that)</t>
+        </is>
+      </c>
+      <c r="L184" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M184" s="3" t="inlineStr">
+        <is>
+          <t>Requirements-Analysis</t>
+        </is>
+      </c>
+      <c r="N184" s="3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="O184" s="3" t="inlineStr">
+        <is>
+          <t>Sanity</t>
+        </is>
+      </c>
+      <c r="P184" s="3" t="inlineStr">
+        <is>
+          <t>EthFw</t>
+        </is>
+      </c>
+      <c r="Q184" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2970</t>
+        </is>
+      </c>
+      <c r="R184" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S184" s="3" t="inlineStr"/>
+      <c r="T184" s="3" t="inlineStr"/>
+      <c r="U184" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2971</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW VLAN test plan</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2878</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>ARP VLAN packets replied by EthFw (proxy arp)</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2895</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="inlineStr">
+        <is>
+          <t>j721e-evm,j7200-evm,j784s4-evm</t>
+        </is>
+      </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="I185" s="3" t="inlineStr">
+        <is>
+          <t>When we send VLAN ARP packet i.e. a VLAN Broadcast packet post a VLAN_JOIN from a client,
+ARP packets reply should come from EthFw.</t>
+        </is>
+      </c>
+      <c r="J185" s="3" t="inlineStr">
+        <is>
+          <t>1. Join VLAN from client (do vlan_join say 1025 from Linux client or add an instruction in RTOS client)
+2. Send a ARP + VLAN of above joined packet to any of switch Port (use packETH)
+3. Check packet receive at ethfw handle ARP rx packet function
+4. Make sure that EthFw replies to this ARP + VLAN
+5. See the reply comes back on external port (use wireshark)</t>
+        </is>
+      </c>
+      <c r="K185" s="3" t="inlineStr">
+        <is>
+          <t>ARP + VLAN packets reply should come from EthFw.</t>
+        </is>
+      </c>
+      <c r="L185" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M185" s="3" t="inlineStr">
+        <is>
+          <t>Requirements-Analysis</t>
+        </is>
+      </c>
+      <c r="N185" s="3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="O185" s="3" t="inlineStr">
+        <is>
+          <t>Sanity</t>
+        </is>
+      </c>
+      <c r="P185" s="3" t="inlineStr">
+        <is>
+          <t>EthFw</t>
+        </is>
+      </c>
+      <c r="Q185" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2970</t>
+        </is>
+      </c>
+      <c r="R185" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S185" s="3" t="inlineStr"/>
+      <c r="T185" s="3" t="inlineStr"/>
+      <c r="U185" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2971</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW VLAN test plan</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2890</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>Exclusive Multicast Address test</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="F186" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2895</t>
+        </is>
+      </c>
+      <c r="G186" s="3" t="inlineStr">
+        <is>
+          <t>j721e-evm,j7200-evm,j784s4-evm</t>
+        </is>
+      </c>
+      <c r="H186" s="3" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="I186" s="3" t="inlineStr">
+        <is>
+          <t>Exclusive multicast address M to be exclusive irrespective of VLAN
+We are stopping other clients to join M post 1 client joins M
+In case when client registers exclusive multicast in a VLAN,
+we are still registering it only at mac address level and ignoring the VLAN provided.</t>
+        </is>
+      </c>
+      <c r="J186" s="3" t="inlineStr">
+        <is>
+          <t>1. Join exclusive multicast from client C (do ip  maddr add from Linux client or add an instruction in RTOS client)
+2. ip maddr add 01:80:c2:00:00:07 dev eth2
+3. Make sure that exclusive multicast gets added
+4. Delete the exclusive mcast addr: ip maddr del 01:80:c2:00:00:07 dev eth2
+5. Make sure that it gets deleted
+6. Do multiple additions from different clients on the same address
+7. Similarly do multiple deletions as well. Make sure you get error on multiple additions and deletions from firmware.</t>
+        </is>
+      </c>
+      <c r="K186" s="3" t="inlineStr">
+        <is>
+          <t>Addition and deletion of exclusive multicast should work fine. Multiple addition or deletion should throw an error.</t>
+        </is>
+      </c>
+      <c r="L186" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M186" s="3" t="inlineStr">
+        <is>
+          <t>Requirements-Analysis</t>
+        </is>
+      </c>
+      <c r="N186" s="3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="O186" s="3" t="inlineStr">
+        <is>
+          <t>Sanity</t>
+        </is>
+      </c>
+      <c r="P186" s="3" t="inlineStr">
+        <is>
+          <t>EthFw</t>
+        </is>
+      </c>
+      <c r="Q186" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW-2970</t>
+        </is>
+      </c>
+      <c r="R186" s="3" t="inlineStr">
+        <is>
+          <t>ETHFW 10.1 Release Test Run (j7200)</t>
+        </is>
+      </c>
+      <c r="S186" s="3" t="inlineStr"/>
+      <c r="T186" s="3" t="inlineStr"/>
+      <c r="U186" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U181"/>
+  <autoFilter ref="A1:U186"/>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
EthFw: 11.2.0: Update release notes and collaterals
- Update release notes, test reports and
  static analysis reports for SDK 11.02.

Fixes: ETHFW-3516
Signed-off-by: Siddharth S <s-s9@ti.com>
</commit_message>
<xml_diff>
--- a/docs/test_report/ethfw_testreport_j7200.xlsx
+++ b/docs/test_report/ethfw_testreport_j7200.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a0512659\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a0512659\Desktop\EthFw 11.2 Collaterals\Test Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7651F4-7D83-4F3C-93B4-A34891189E9B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A4F04F2-96D9-4A96-ACD9-13685808D65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11505" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table of Contents" sheetId="1" r:id="rId1"/>
@@ -105,13 +105,13 @@
     <t>Report generated on</t>
   </si>
   <si>
-    <t>ETHFW-3388</t>
+    <t>ETHFW-3507</t>
   </si>
   <si>
     <t>None</t>
   </si>
   <si>
-    <t>2025-08-21 06:17:10.456604-05:00 CDT</t>
+    <t>2025-12-09 05:50:16.097896-06:00 CDT</t>
   </si>
   <si>
     <t>Test Level | Overall Status</t>
@@ -141,10 +141,10 @@
     <t>0</t>
   </si>
   <si>
-    <t>78</t>
-  </si>
-  <si>
-    <t>2</t>
+    <t>76</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
   <si>
     <t>80</t>
@@ -162,10 +162,10 @@
     <t>Validation</t>
   </si>
   <si>
-    <t>103</t>
-  </si>
-  <si>
-    <t>3</t>
+    <t>105</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
   <si>
     <t>106</t>
@@ -189,19 +189,19 @@
     <t>0%</t>
   </si>
   <si>
-    <t>98%</t>
-  </si>
-  <si>
-    <t>2%</t>
+    <t>95%</t>
+  </si>
+  <si>
+    <t>5%</t>
   </si>
   <si>
     <t>100%</t>
   </si>
   <si>
-    <t>97%</t>
-  </si>
-  <si>
-    <t>3%</t>
+    <t>99%</t>
+  </si>
+  <si>
+    <t>1%</t>
   </si>
   <si>
     <t>Test Type</t>
@@ -333,7 +333,7 @@
     <t>EthFw</t>
   </si>
   <si>
-    <t>ETHFW 11.1 Release Test Run (j7200)</t>
+    <t>ETHFW 11.2 Release Test Run (j7200)</t>
   </si>
   <si>
     <t>ETHFW-1010</t>
@@ -3728,16 +3728,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3779,12 +3777,6 @@
         <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -3813,7 +3805,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3843,9 +3835,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4180,18 +4169,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -6698,7 +6687,7 @@
       <c r="T31" s="1" t="s">
         <v>1043</v>
       </c>
-      <c r="U31" s="11" t="s">
+      <c r="U31" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -9874,7 +9863,7 @@
       <c r="T83" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="U83" s="11" t="s">
+      <c r="U83" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -10244,7 +10233,7 @@
       <c r="T89" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="U89" s="11" t="s">
+      <c r="U89" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -15860,7 +15849,7 @@
       <c r="T181" s="1" t="s">
         <v>891</v>
       </c>
-      <c r="U181" s="11" t="s">
+      <c r="U181" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -16574,7 +16563,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>960</v>
       </c>
       <c r="B2" s="10" t="s">
@@ -16591,7 +16580,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
+      <c r="A3" s="17"/>
       <c r="B3" s="10" t="s">
         <v>68</v>
       </c>
@@ -16606,7 +16595,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="18"/>
+      <c r="A4" s="17"/>
       <c r="B4" s="10" t="s">
         <v>69</v>
       </c>
@@ -16621,7 +16610,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
+      <c r="A5" s="17"/>
       <c r="B5" s="10" t="s">
         <v>70</v>
       </c>
@@ -16636,7 +16625,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="120" x14ac:dyDescent="0.25">
-      <c r="A6" s="18"/>
+      <c r="A6" s="17"/>
       <c r="B6" s="10" t="s">
         <v>71</v>
       </c>
@@ -16651,7 +16640,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="18"/>
+      <c r="A7" s="17"/>
       <c r="B7" s="10" t="s">
         <v>72</v>
       </c>
@@ -16666,7 +16655,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="18"/>
+      <c r="A8" s="17"/>
       <c r="B8" s="10" t="s">
         <v>968</v>
       </c>
@@ -16681,7 +16670,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="120" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
+      <c r="A9" s="17"/>
       <c r="B9" s="10" t="s">
         <v>74</v>
       </c>
@@ -16696,7 +16685,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="18"/>
+      <c r="A10" s="17"/>
       <c r="B10" s="10" t="s">
         <v>75</v>
       </c>
@@ -16711,7 +16700,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="18"/>
+      <c r="A11" s="17"/>
       <c r="B11" s="10" t="s">
         <v>76</v>
       </c>
@@ -16726,7 +16715,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="18"/>
+      <c r="A12" s="17"/>
       <c r="B12" s="10" t="s">
         <v>77</v>
       </c>
@@ -16741,8 +16730,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A13" s="18"/>
-      <c r="B13" s="17" t="s">
+      <c r="A13" s="17"/>
+      <c r="B13" s="16" t="s">
         <v>57</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -16756,8 +16745,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="18"/>
-      <c r="B14" s="17"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="1" t="s">
         <v>976</v>
       </c>
@@ -16769,8 +16758,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="105" x14ac:dyDescent="0.25">
-      <c r="A15" s="18"/>
-      <c r="B15" s="17"/>
+      <c r="A15" s="17"/>
+      <c r="B15" s="16"/>
       <c r="C15" s="1" t="s">
         <v>977</v>
       </c>
@@ -16782,8 +16771,8 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="18"/>
-      <c r="B16" s="17"/>
+      <c r="A16" s="17"/>
+      <c r="B16" s="16"/>
       <c r="C16" s="1" t="s">
         <v>978</v>
       </c>
@@ -16795,8 +16784,8 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="18"/>
-      <c r="B17" s="17"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="1" t="s">
         <v>979</v>
       </c>
@@ -16808,8 +16797,8 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="18"/>
-      <c r="B18" s="17"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="1" t="s">
         <v>980</v>
       </c>
@@ -16821,8 +16810,8 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A19" s="18"/>
-      <c r="B19" s="17"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="16"/>
       <c r="C19" s="1" t="s">
         <v>981</v>
       </c>
@@ -16834,8 +16823,8 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="105" x14ac:dyDescent="0.25">
-      <c r="A20" s="18"/>
-      <c r="B20" s="17"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="16"/>
       <c r="C20" s="1" t="s">
         <v>982</v>
       </c>
@@ -16847,8 +16836,8 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="135" x14ac:dyDescent="0.25">
-      <c r="A21" s="18"/>
-      <c r="B21" s="17"/>
+      <c r="A21" s="17"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="1" t="s">
         <v>983</v>
       </c>
@@ -16860,8 +16849,8 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A22" s="18"/>
-      <c r="B22" s="17"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="1" t="s">
         <v>984</v>
       </c>
@@ -16873,8 +16862,8 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="105" x14ac:dyDescent="0.25">
-      <c r="A23" s="18"/>
-      <c r="B23" s="17"/>
+      <c r="A23" s="17"/>
+      <c r="B23" s="16"/>
       <c r="C23" s="1" t="s">
         <v>985</v>
       </c>
@@ -16886,8 +16875,8 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="180" x14ac:dyDescent="0.25">
-      <c r="A24" s="18"/>
-      <c r="B24" s="17" t="s">
+      <c r="A24" s="17"/>
+      <c r="B24" s="16" t="s">
         <v>986</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -16901,8 +16890,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A25" s="18"/>
-      <c r="B25" s="17"/>
+      <c r="A25" s="17"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="1" t="s">
         <v>988</v>
       </c>
@@ -16914,8 +16903,8 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="18"/>
-      <c r="B26" s="17"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="1" t="s">
         <v>989</v>
       </c>
@@ -16927,8 +16916,8 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A27" s="18"/>
-      <c r="B27" s="17"/>
+      <c r="A27" s="17"/>
+      <c r="B27" s="16"/>
       <c r="C27" s="1" t="s">
         <v>990</v>
       </c>
@@ -16940,8 +16929,8 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A28" s="18"/>
-      <c r="B28" s="17"/>
+      <c r="A28" s="17"/>
+      <c r="B28" s="16"/>
       <c r="C28" s="1" t="s">
         <v>991</v>
       </c>
@@ -16953,7 +16942,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="18"/>
+      <c r="A29" s="17"/>
       <c r="B29" s="10" t="s">
         <v>79</v>
       </c>
@@ -16968,8 +16957,8 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="18"/>
-      <c r="B30" s="17" t="s">
+      <c r="A30" s="17"/>
+      <c r="B30" s="16" t="s">
         <v>80</v>
       </c>
       <c r="C30" s="1" t="s">
@@ -16983,8 +16972,8 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A31" s="18"/>
-      <c r="B31" s="17"/>
+      <c r="A31" s="17"/>
+      <c r="B31" s="16"/>
       <c r="C31" s="1" t="s">
         <v>994</v>
       </c>
@@ -16996,8 +16985,8 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="18"/>
-      <c r="B32" s="17"/>
+      <c r="A32" s="17"/>
+      <c r="B32" s="16"/>
       <c r="C32" s="1" t="s">
         <v>995</v>
       </c>
@@ -17009,8 +16998,8 @@
       </c>
     </row>
     <row r="33" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A33" s="18"/>
-      <c r="B33" s="17"/>
+      <c r="A33" s="17"/>
+      <c r="B33" s="16"/>
       <c r="C33" s="1" t="s">
         <v>996</v>
       </c>
@@ -17022,7 +17011,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="18"/>
+      <c r="A34" s="17"/>
       <c r="B34" s="10" t="s">
         <v>81</v>
       </c>
@@ -17037,7 +17026,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="15" t="s">
         <v>998</v>
       </c>
       <c r="B35" s="10" t="s">
@@ -17054,7 +17043,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="16"/>
+      <c r="A36" s="15"/>
       <c r="B36" s="10" t="s">
         <v>84</v>
       </c>
@@ -17069,7 +17058,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="16"/>
+      <c r="A37" s="15"/>
       <c r="B37" s="10" t="s">
         <v>85</v>
       </c>
@@ -17084,8 +17073,8 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="16"/>
-      <c r="B38" s="17" t="s">
+      <c r="A38" s="15"/>
+      <c r="B38" s="16" t="s">
         <v>86</v>
       </c>
       <c r="C38" s="1" t="s">
@@ -17099,8 +17088,8 @@
       </c>
     </row>
     <row r="39" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A39" s="16"/>
-      <c r="B39" s="17"/>
+      <c r="A39" s="15"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="1" t="s">
         <v>1003</v>
       </c>
@@ -17112,8 +17101,8 @@
       </c>
     </row>
     <row r="40" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
-      <c r="B40" s="17"/>
+      <c r="A40" s="15"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="1" t="s">
         <v>1004</v>
       </c>
@@ -17125,8 +17114,8 @@
       </c>
     </row>
     <row r="41" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
-      <c r="B41" s="17"/>
+      <c r="A41" s="15"/>
+      <c r="B41" s="16"/>
       <c r="C41" s="1" t="s">
         <v>1005</v>
       </c>
@@ -17138,8 +17127,8 @@
       </c>
     </row>
     <row r="42" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
-      <c r="B42" s="17"/>
+      <c r="A42" s="15"/>
+      <c r="B42" s="16"/>
       <c r="C42" s="1" t="s">
         <v>1006</v>
       </c>

</xml_diff>